<commit_message>
Update NVDA data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/NVDA_data.xlsx
+++ b/data/NVDA_data.xlsx
@@ -4764,7 +4764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4885,25 +4885,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -4963,7 +4983,7 @@
         <v>2.217</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -4987,29 +5007,41 @@
       <c r="W2" t="n">
         <v>4.589</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>9.483000000000001</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>24.291891</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1.278</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>24147000000</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Semiconductors</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.nvidia.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>NVIDIA Corporation operates as a data center scale AI infrastructure company in the United States, Taiwan, China, Hong Kong, Europe, and internationally. It operates through Compute &amp; Networking, and Graphics segments. The Compute &amp; Networking segment provides data center accelerated computing and networking platforms and artificial intelligence solutions and software, and automotive platforms and autonomous and electric vehicle solutions, including software. The Graphics segment offers GeForce GPUs for gaming and PCs; Quadro/NVIDIA RTX GPUs for enterprise workstation graphics. The company's products are used in gaming, professional visualization, data center, and automotive markets. It sells its products to original equipment manufacturers, original device manufacturers, system integrators and distributors, independent software vendors, cloud service providers, add-in board manufacturers, distributors, automotive manufacturers and tier-1 automotive suppliers, and other ecosystem participants. NVIDIA Corporation was incorporated in 1993 and is headquartered in Santa Clara, California.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:41:56</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:09:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NVDA data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/NVDA_data.xlsx
+++ b/data/NVDA_data.xlsx
@@ -4985,15 +4985,11 @@
       <c r="Q2" t="n">
         <v>0.43</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.63663</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.66236997</v>
       </c>
       <c r="T2" t="n">
         <v>1.17211</v>
@@ -5041,7 +5037,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:49:03</t>
+          <t>2026-09-06 16:59:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NVDA data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/NVDA_data.xlsx
+++ b/data/NVDA_data.xlsx
@@ -4764,7 +4764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4905,25 +4905,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5015,29 +5030,38 @@
       <c r="AA2" t="n">
         <v>24147000000</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>302970011648</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>5528066981888</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>201266003968</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Semiconductors</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.nvidia.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>NVIDIA Corporation operates as a data center scale AI infrastructure company in the United States, Taiwan, China, Hong Kong, Europe, and internationally. It operates through Compute &amp; Networking, and Graphics segments. The Compute &amp; Networking segment provides data center accelerated computing and networking platforms and artificial intelligence solutions and software, and automotive platforms and autonomous and electric vehicle solutions, including software. The Graphics segment offers GeForce GPUs for gaming and PCs; Quadro/NVIDIA RTX GPUs for enterprise workstation graphics. The company's products are used in gaming, professional visualization, data center, and automotive markets. It sells its products to original equipment manufacturers, original device manufacturers, system integrators and distributors, independent software vendors, cloud service providers, add-in board manufacturers, distributors, automotive manufacturers and tier-1 automotive suppliers, and other ecosystem participants. NVIDIA Corporation was incorporated in 1993 and is headquartered in Santa Clara, California.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:34</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NVDA data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/NVDA_data.xlsx
+++ b/data/NVDA_data.xlsx
@@ -472,16 +472,16 @@
         <v>45905</v>
       </c>
       <c r="B2" t="n">
-        <v>167.8065180303181</v>
+        <v>167.8065026792569</v>
       </c>
       <c r="C2" t="n">
-        <v>168.8051880252559</v>
+        <v>168.8051725828357</v>
       </c>
       <c r="D2" t="n">
-        <v>163.8517933839215</v>
+        <v>163.8517783946414</v>
       </c>
       <c r="E2" t="n">
-        <v>166.7978668212891</v>
+        <v>166.7978515625</v>
       </c>
       <c r="F2" t="n">
         <v>224441400</v>
@@ -498,16 +498,16 @@
         <v>45908</v>
       </c>
       <c r="B3" t="n">
-        <v>167.3271370026614</v>
+        <v>167.3271521925502</v>
       </c>
       <c r="C3" t="n">
-        <v>170.7326048603557</v>
+        <v>170.7326203593915</v>
       </c>
       <c r="D3" t="n">
-        <v>167.1274060796587</v>
+        <v>167.127421251416</v>
       </c>
       <c r="E3" t="n">
-        <v>168.0861206054688</v>
+        <v>168.0861358642578</v>
       </c>
       <c r="F3" t="n">
         <v>163769100</v>
@@ -524,16 +524,16 @@
         <v>45909</v>
       </c>
       <c r="B4" t="n">
-        <v>168.8650754099384</v>
+        <v>168.8650905194996</v>
       </c>
       <c r="C4" t="n">
-        <v>170.7525607512945</v>
+        <v>170.7525760297424</v>
       </c>
       <c r="D4" t="n">
-        <v>166.518210487105</v>
+        <v>166.5182253866755</v>
       </c>
       <c r="E4" t="n">
-        <v>170.5328521728516</v>
+        <v>170.5328674316406</v>
       </c>
       <c r="F4" t="n">
         <v>157548400</v>
@@ -550,16 +550,16 @@
         <v>45910</v>
       </c>
       <c r="B5" t="n">
-        <v>176.4050468150653</v>
+        <v>176.4050620144814</v>
       </c>
       <c r="C5" t="n">
-        <v>179.0515158989888</v>
+        <v>179.05153132643</v>
       </c>
       <c r="D5" t="n">
-        <v>175.2366048852674</v>
+        <v>175.2366199840082</v>
       </c>
       <c r="E5" t="n">
-        <v>177.0941314697266</v>
+        <v>177.0941467285156</v>
       </c>
       <c r="F5" t="n">
         <v>226852000</v>
@@ -576,16 +576,16 @@
         <v>45911</v>
       </c>
       <c r="B6" t="n">
-        <v>179.4511334529312</v>
+        <v>179.4511025030058</v>
       </c>
       <c r="C6" t="n">
-        <v>180.0503753259473</v>
+        <v>180.0503442726707</v>
       </c>
       <c r="D6" t="n">
-        <v>176.2552123553376</v>
+        <v>176.2551819566126</v>
       </c>
       <c r="E6" t="n">
-        <v>176.9443359375</v>
+        <v>176.9443054199219</v>
       </c>
       <c r="F6" t="n">
         <v>151159300</v>
@@ -602,16 +602,16 @@
         <v>45912</v>
       </c>
       <c r="B7" t="n">
-        <v>177.5435512454145</v>
+        <v>177.5435664999128</v>
       </c>
       <c r="C7" t="n">
-        <v>178.3724957753353</v>
+        <v>178.3725111010563</v>
       </c>
       <c r="D7" t="n">
-        <v>176.2252254177762</v>
+        <v>176.2252405590043</v>
       </c>
       <c r="E7" t="n">
-        <v>177.5934906005859</v>
+        <v>177.593505859375</v>
       </c>
       <c r="F7" t="n">
         <v>124911000</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>175.4462376691102</v>
+        <v>175.446222588877</v>
       </c>
       <c r="C8" t="n">
-        <v>178.6221950533741</v>
+        <v>178.622179700156</v>
       </c>
       <c r="D8" t="n">
-        <v>174.28771156721</v>
+        <v>174.2876965865563</v>
       </c>
       <c r="E8" t="n">
-        <v>177.5235900878906</v>
+        <v>177.5235748291016</v>
       </c>
       <c r="F8" t="n">
         <v>147061600</v>
@@ -758,16 +758,16 @@
         <v>45922</v>
       </c>
       <c r="B13" t="n">
-        <v>175.0767018025102</v>
+        <v>175.0767163707024</v>
       </c>
       <c r="C13" t="n">
-        <v>184.314918935884</v>
+        <v>184.3149342727913</v>
       </c>
       <c r="D13" t="n">
-        <v>174.487457015772</v>
+        <v>174.4874715349329</v>
       </c>
       <c r="E13" t="n">
-        <v>183.3761138916016</v>
+        <v>183.3761291503906</v>
       </c>
       <c r="F13" t="n">
         <v>269637000</v>
@@ -888,16 +888,16 @@
         <v>45929</v>
       </c>
       <c r="B18" t="n">
-        <v>180.2001729762767</v>
+        <v>180.2001578366391</v>
       </c>
       <c r="C18" t="n">
-        <v>183.7656330630971</v>
+        <v>183.765617623905</v>
       </c>
       <c r="D18" t="n">
-        <v>180.0903277167248</v>
+        <v>180.0903125863159</v>
       </c>
       <c r="E18" t="n">
-        <v>181.6183776855469</v>
+        <v>181.6183624267578</v>
       </c>
       <c r="F18" t="n">
         <v>193063500</v>
@@ -940,16 +940,16 @@
         <v>45931</v>
       </c>
       <c r="B20" t="n">
-        <v>185.0040430020549</v>
+        <v>185.0040580978575</v>
       </c>
       <c r="C20" t="n">
-        <v>187.9003428272602</v>
+        <v>187.9003581593927</v>
       </c>
       <c r="D20" t="n">
-        <v>183.6657383394342</v>
+        <v>183.665753326035</v>
       </c>
       <c r="E20" t="n">
-        <v>187.0014953613281</v>
+        <v>187.0015106201172</v>
       </c>
       <c r="F20" t="n">
         <v>173844900</v>
@@ -992,16 +992,16 @@
         <v>45933</v>
       </c>
       <c r="B22" t="n">
-        <v>188.9490194719917</v>
+        <v>188.9490040855168</v>
       </c>
       <c r="C22" t="n">
-        <v>190.1175273421404</v>
+        <v>190.1175118605118</v>
       </c>
       <c r="D22" t="n">
-        <v>185.1438749421695</v>
+        <v>185.1438598655547</v>
       </c>
       <c r="E22" t="n">
-        <v>187.3810119628906</v>
+        <v>187.3809967041016</v>
       </c>
       <c r="F22" t="n">
         <v>137596900</v>
@@ -1018,16 +1018,16 @@
         <v>45936</v>
       </c>
       <c r="B23" t="n">
-        <v>185.2637075602064</v>
+        <v>185.2637228157064</v>
       </c>
       <c r="C23" t="n">
-        <v>186.9914995955013</v>
+        <v>186.991514993276</v>
       </c>
       <c r="D23" t="n">
-        <v>183.0964735646395</v>
+        <v>183.0964886416791</v>
       </c>
       <c r="E23" t="n">
-        <v>185.3036499023438</v>
+        <v>185.3036651611328</v>
       </c>
       <c r="F23" t="n">
         <v>157678100</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>187.7305636382236</v>
+        <v>187.7305788686531</v>
       </c>
       <c r="C28" t="n">
-        <v>189.8678370807686</v>
+        <v>189.8678524845934</v>
       </c>
       <c r="D28" t="n">
-        <v>185.7231294773067</v>
+        <v>185.7231445448746</v>
       </c>
       <c r="E28" t="n">
-        <v>188.0801239013672</v>
+        <v>188.0801391601562</v>
       </c>
       <c r="F28" t="n">
         <v>153482800</v>
@@ -1174,16 +1174,16 @@
         <v>45944</v>
       </c>
       <c r="B29" t="n">
-        <v>184.5346263960681</v>
+        <v>184.5346420566055</v>
       </c>
       <c r="C29" t="n">
-        <v>184.5645869600227</v>
+        <v>184.5646026231026</v>
       </c>
       <c r="D29" t="n">
-        <v>179.4710777368365</v>
+        <v>179.4710929676557</v>
       </c>
       <c r="E29" t="n">
-        <v>179.8006591796875</v>
+        <v>179.8006744384766</v>
       </c>
       <c r="F29" t="n">
         <v>205641400</v>
@@ -1226,16 +1226,16 @@
         <v>45946</v>
       </c>
       <c r="B31" t="n">
-        <v>181.9978781082864</v>
+        <v>181.9978628142482</v>
       </c>
       <c r="C31" t="n">
-        <v>183.0465437061986</v>
+        <v>183.0465283240366</v>
       </c>
       <c r="D31" t="n">
-        <v>179.5410200965125</v>
+        <v>179.5410050089342</v>
       </c>
       <c r="E31" t="n">
-        <v>181.5784149169922</v>
+        <v>181.5783996582031</v>
       </c>
       <c r="F31" t="n">
         <v>179723300</v>
@@ -1304,16 +1304,16 @@
         <v>45951</v>
       </c>
       <c r="B34" t="n">
-        <v>182.5571429687811</v>
+        <v>182.5571583648613</v>
       </c>
       <c r="C34" t="n">
-        <v>182.5571429687811</v>
+        <v>182.5571583648613</v>
       </c>
       <c r="D34" t="n">
-        <v>179.5709615871908</v>
+        <v>179.5709767314294</v>
       </c>
       <c r="E34" t="n">
-        <v>180.9292297363281</v>
+        <v>180.9292449951172</v>
       </c>
       <c r="F34" t="n">
         <v>124240200</v>
@@ -1382,16 +1382,16 @@
         <v>45954</v>
       </c>
       <c r="B37" t="n">
-        <v>183.6058049719722</v>
+        <v>183.6058200325102</v>
       </c>
       <c r="C37" t="n">
-        <v>187.2311856390606</v>
+        <v>187.2312009969758</v>
       </c>
       <c r="D37" t="n">
-        <v>183.2662417509678</v>
+        <v>183.2662567836526</v>
       </c>
       <c r="E37" t="n">
-        <v>186.0227203369141</v>
+        <v>186.0227355957031</v>
       </c>
       <c r="F37" t="n">
         <v>131296700</v>
@@ -1408,16 +1408,16 @@
         <v>45957</v>
       </c>
       <c r="B38" t="n">
-        <v>189.7479892463022</v>
+        <v>189.7480043855645</v>
       </c>
       <c r="C38" t="n">
-        <v>191.7554233483132</v>
+        <v>191.755438647741</v>
       </c>
       <c r="D38" t="n">
-        <v>188.1899636305417</v>
+        <v>188.189978645495</v>
       </c>
       <c r="E38" t="n">
-        <v>191.2460784912109</v>
+        <v>191.24609375</v>
       </c>
       <c r="F38" t="n">
         <v>153452700</v>
@@ -1434,16 +1434,16 @@
         <v>45958</v>
       </c>
       <c r="B39" t="n">
-        <v>192.8041096644758</v>
+        <v>192.8040950113927</v>
       </c>
       <c r="C39" t="n">
-        <v>202.8912358579665</v>
+        <v>202.8912204382634</v>
       </c>
       <c r="D39" t="n">
-        <v>191.6655623251096</v>
+        <v>191.6655477585559</v>
       </c>
       <c r="E39" t="n">
-        <v>200.7739410400391</v>
+        <v>200.77392578125</v>
       </c>
       <c r="F39" t="n">
         <v>297986200</v>
@@ -1538,16 +1538,16 @@
         <v>45964</v>
       </c>
       <c r="B43" t="n">
-        <v>207.8149386664238</v>
+        <v>207.8149540137207</v>
       </c>
       <c r="C43" t="n">
-        <v>211.0707804221397</v>
+        <v>211.0707960098831</v>
       </c>
       <c r="D43" t="n">
-        <v>205.2981445069072</v>
+        <v>205.2981596683369</v>
       </c>
       <c r="E43" t="n">
-        <v>206.6164703369141</v>
+        <v>206.6164855957031</v>
       </c>
       <c r="F43" t="n">
         <v>180267300</v>
@@ -1616,16 +1616,16 @@
         <v>45967</v>
       </c>
       <c r="B46" t="n">
-        <v>196.169796348482</v>
+        <v>196.1698122838887</v>
       </c>
       <c r="C46" t="n">
-        <v>197.3682647282291</v>
+        <v>197.3682807609907</v>
       </c>
       <c r="D46" t="n">
-        <v>186.1425921093966</v>
+        <v>186.1426072302662</v>
       </c>
       <c r="E46" t="n">
-        <v>187.8404235839844</v>
+        <v>187.8404388427734</v>
       </c>
       <c r="F46" t="n">
         <v>223029800</v>
@@ -1642,16 +1642,16 @@
         <v>45968</v>
       </c>
       <c r="B47" t="n">
-        <v>184.6644790168218</v>
+        <v>184.6644490263876</v>
       </c>
       <c r="C47" t="n">
-        <v>188.0801362299674</v>
+        <v>188.0801056848134</v>
       </c>
       <c r="D47" t="n">
-        <v>178.682118484317</v>
+        <v>178.682089465448</v>
       </c>
       <c r="E47" t="n">
-        <v>187.9103393554688</v>
+        <v>187.9103088378906</v>
       </c>
       <c r="F47" t="n">
         <v>264942300</v>
@@ -1720,16 +1720,16 @@
         <v>45973</v>
       </c>
       <c r="B50" t="n">
-        <v>195.4706988945922</v>
+        <v>195.4706834846326</v>
       </c>
       <c r="C50" t="n">
-        <v>195.6404805249176</v>
+        <v>195.6404651015733</v>
       </c>
       <c r="D50" t="n">
-        <v>190.8865491577477</v>
+        <v>190.8865341091802</v>
       </c>
       <c r="E50" t="n">
-        <v>193.5531463623047</v>
+        <v>193.5531311035156</v>
       </c>
       <c r="F50" t="n">
         <v>154935300</v>
@@ -1746,16 +1746,16 @@
         <v>45974</v>
       </c>
       <c r="B51" t="n">
-        <v>190.806628384499</v>
+        <v>190.8066439854392</v>
       </c>
       <c r="C51" t="n">
-        <v>191.1961309619508</v>
+        <v>191.1961465947379</v>
       </c>
       <c r="D51" t="n">
-        <v>183.6158033642</v>
+        <v>183.6158183771961</v>
       </c>
       <c r="E51" t="n">
-        <v>186.6219635009766</v>
+        <v>186.6219787597656</v>
       </c>
       <c r="F51" t="n">
         <v>207423100</v>
@@ -1798,16 +1798,16 @@
         <v>45978</v>
       </c>
       <c r="B53" t="n">
-        <v>185.7331023397778</v>
+        <v>185.7331175470496</v>
       </c>
       <c r="C53" t="n">
-        <v>188.7592413389203</v>
+        <v>188.7592567939633</v>
       </c>
       <c r="D53" t="n">
-        <v>184.0852102968453</v>
+        <v>184.0852253691927</v>
       </c>
       <c r="E53" t="n">
-        <v>186.3623046875</v>
+        <v>186.3623199462891</v>
       </c>
       <c r="F53" t="n">
         <v>173628900</v>
@@ -1824,16 +1824,16 @@
         <v>45979</v>
       </c>
       <c r="B54" t="n">
-        <v>183.1464137160556</v>
+        <v>183.1464291447985</v>
       </c>
       <c r="C54" t="n">
-        <v>184.5646030780414</v>
+        <v>184.5646186262563</v>
       </c>
       <c r="D54" t="n">
-        <v>179.4211540526368</v>
+        <v>179.4211691675539</v>
       </c>
       <c r="E54" t="n">
-        <v>181.1289825439453</v>
+        <v>181.1289978027344</v>
       </c>
       <c r="F54" t="n">
         <v>213598900</v>
@@ -1954,16 +1954,16 @@
         <v>45986</v>
       </c>
       <c r="B59" t="n">
-        <v>174.6871938582165</v>
+        <v>174.6872088672972</v>
       </c>
       <c r="C59" t="n">
-        <v>177.9330538327892</v>
+        <v>177.9330691207534</v>
       </c>
       <c r="D59" t="n">
-        <v>169.3340211059625</v>
+        <v>169.3340356551</v>
       </c>
       <c r="E59" t="n">
-        <v>177.5934906005859</v>
+        <v>177.593505859375</v>
       </c>
       <c r="F59" t="n">
         <v>320600300</v>
@@ -1980,16 +1980,16 @@
         <v>45987</v>
       </c>
       <c r="B60" t="n">
-        <v>181.3986455127995</v>
+        <v>181.3986301380407</v>
       </c>
       <c r="C60" t="n">
-        <v>182.6770138362068</v>
+        <v>182.6769983530976</v>
       </c>
       <c r="D60" t="n">
-        <v>178.0129642870119</v>
+        <v>178.0129491992125</v>
       </c>
       <c r="E60" t="n">
-        <v>180.0303802490234</v>
+        <v>180.0303649902344</v>
       </c>
       <c r="F60" t="n">
         <v>183852000</v>
@@ -2032,16 +2032,16 @@
         <v>45992</v>
       </c>
       <c r="B62" t="n">
-        <v>174.5373952700045</v>
+        <v>174.5373804488289</v>
       </c>
       <c r="C62" t="n">
-        <v>180.0703472704488</v>
+        <v>180.070331979432</v>
       </c>
       <c r="D62" t="n">
-        <v>173.4587690832101</v>
+        <v>173.4587543536281</v>
       </c>
       <c r="E62" t="n">
-        <v>179.6908264160156</v>
+        <v>179.6908111572266</v>
       </c>
       <c r="F62" t="n">
         <v>188131000</v>
@@ -2058,16 +2058,16 @@
         <v>45993</v>
       </c>
       <c r="B63" t="n">
-        <v>181.528456967636</v>
+        <v>181.5284722516508</v>
       </c>
       <c r="C63" t="n">
-        <v>185.4234980410985</v>
+        <v>185.4235136530611</v>
       </c>
       <c r="D63" t="n">
-        <v>179.77070445469</v>
+        <v>179.7707195907086</v>
       </c>
       <c r="E63" t="n">
-        <v>181.2288513183594</v>
+        <v>181.2288665771484</v>
       </c>
       <c r="F63" t="n">
         <v>182632200</v>
@@ -2084,16 +2084,16 @@
         <v>45994</v>
       </c>
       <c r="B64" t="n">
-        <v>180.8493441127912</v>
+        <v>180.849359498178</v>
       </c>
       <c r="C64" t="n">
-        <v>182.2175941452395</v>
+        <v>182.2176096470274</v>
       </c>
       <c r="D64" t="n">
-        <v>178.8818522580144</v>
+        <v>178.8818674760209</v>
       </c>
       <c r="E64" t="n">
-        <v>179.3612365722656</v>
+        <v>179.3612518310547</v>
       </c>
       <c r="F64" t="n">
         <v>165138000</v>
@@ -2110,16 +2110,16 @@
         <v>45995</v>
       </c>
       <c r="B65" t="n">
-        <v>181.3987504426599</v>
+        <v>181.3987353303187</v>
       </c>
       <c r="C65" t="n">
-        <v>184.2952268834804</v>
+        <v>184.2952115298336</v>
       </c>
       <c r="D65" t="n">
-        <v>179.7407841933088</v>
+        <v>179.7407692190929</v>
       </c>
       <c r="E65" t="n">
-        <v>183.1566162109375</v>
+        <v>183.1566009521484</v>
       </c>
       <c r="F65" t="n">
         <v>167364900</v>
@@ -2292,16 +2292,16 @@
         <v>46006</v>
       </c>
       <c r="B72" t="n">
-        <v>177.7232402429772</v>
+        <v>177.7232248413715</v>
       </c>
       <c r="C72" t="n">
-        <v>178.2026512513541</v>
+        <v>178.2026358082024</v>
       </c>
       <c r="D72" t="n">
-        <v>174.8167814768023</v>
+        <v>174.8167663270721</v>
       </c>
       <c r="E72" t="n">
-        <v>176.0752410888672</v>
+        <v>176.0752258300781</v>
       </c>
       <c r="F72" t="n">
         <v>164775600</v>
@@ -2318,16 +2318,16 @@
         <v>46007</v>
       </c>
       <c r="B73" t="n">
-        <v>176.0452813318811</v>
+        <v>176.0452661984462</v>
       </c>
       <c r="C73" t="n">
-        <v>178.27257580423</v>
+        <v>178.2725604793295</v>
       </c>
       <c r="D73" t="n">
-        <v>174.6869374221882</v>
+        <v>174.686922405521</v>
       </c>
       <c r="E73" t="n">
-        <v>177.5035095214844</v>
+        <v>177.5034942626953</v>
       </c>
       <c r="F73" t="n">
         <v>148588100</v>
@@ -2344,16 +2344,16 @@
         <v>46008</v>
       </c>
       <c r="B74" t="n">
-        <v>175.8854835656673</v>
+        <v>175.8854678462756</v>
       </c>
       <c r="C74" t="n">
-        <v>175.9154458008753</v>
+        <v>175.9154300788059</v>
       </c>
       <c r="D74" t="n">
-        <v>170.1025283272995</v>
+        <v>170.1025131247471</v>
       </c>
       <c r="E74" t="n">
-        <v>170.7317657470703</v>
+        <v>170.7317504882812</v>
       </c>
       <c r="F74" t="n">
         <v>222775500</v>
@@ -2396,16 +2396,16 @@
         <v>46010</v>
       </c>
       <c r="B76" t="n">
-        <v>176.4547714783875</v>
+        <v>176.4547863729682</v>
       </c>
       <c r="C76" t="n">
-        <v>181.2289470656948</v>
+        <v>181.2289623632645</v>
       </c>
       <c r="D76" t="n">
-        <v>176.1251716691968</v>
+        <v>176.1251865359559</v>
       </c>
       <c r="E76" t="n">
-        <v>180.7695159912109</v>
+        <v>180.76953125</v>
       </c>
       <c r="F76" t="n">
         <v>324925900</v>
@@ -2448,16 +2448,16 @@
         <v>46014</v>
       </c>
       <c r="B78" t="n">
-        <v>182.7471036477755</v>
+        <v>182.747118403341</v>
       </c>
       <c r="C78" t="n">
-        <v>189.099356383118</v>
+        <v>189.099371651584</v>
       </c>
       <c r="D78" t="n">
-        <v>182.6771816078249</v>
+        <v>182.6771963577447</v>
       </c>
       <c r="E78" t="n">
-        <v>188.9795074462891</v>
+        <v>188.9795227050781</v>
       </c>
       <c r="F78" t="n">
         <v>174873600</v>
@@ -2578,16 +2578,16 @@
         <v>46022</v>
       </c>
       <c r="B83" t="n">
-        <v>189.3390794328336</v>
+        <v>189.3390639228672</v>
       </c>
       <c r="C83" t="n">
-        <v>190.3278636939614</v>
+        <v>190.3278481029973</v>
       </c>
       <c r="D83" t="n">
-        <v>186.262829557789</v>
+        <v>186.2628142998177</v>
       </c>
       <c r="E83" t="n">
-        <v>186.2728118896484</v>
+        <v>186.2727966308594</v>
       </c>
       <c r="F83" t="n">
         <v>120100500</v>
@@ -2708,16 +2708,16 @@
         <v>46030</v>
       </c>
       <c r="B88" t="n">
-        <v>188.8796399788686</v>
+        <v>188.8796243844581</v>
       </c>
       <c r="C88" t="n">
-        <v>189.3191064399463</v>
+        <v>189.3190908092523</v>
       </c>
       <c r="D88" t="n">
-        <v>183.4862239788465</v>
+        <v>183.4862088297309</v>
       </c>
       <c r="E88" t="n">
-        <v>184.8145904541016</v>
+        <v>184.8145751953125</v>
       </c>
       <c r="F88" t="n">
         <v>172457000</v>
@@ -2812,16 +2812,16 @@
         <v>46036</v>
       </c>
       <c r="B92" t="n">
-        <v>184.0954557419801</v>
+        <v>184.0954710990846</v>
       </c>
       <c r="C92" t="n">
-        <v>184.2352845745365</v>
+        <v>184.2352999433054</v>
       </c>
       <c r="D92" t="n">
-        <v>180.5797397860201</v>
+        <v>180.5797548498462</v>
       </c>
       <c r="E92" t="n">
-        <v>182.9168853759766</v>
+        <v>182.9169006347656</v>
       </c>
       <c r="F92" t="n">
         <v>159586100</v>
@@ -2838,16 +2838,16 @@
         <v>46037</v>
       </c>
       <c r="B93" t="n">
-        <v>186.2728105024844</v>
+        <v>186.2727952885624</v>
       </c>
       <c r="C93" t="n">
-        <v>189.4689092968461</v>
+        <v>189.4688938218812</v>
       </c>
       <c r="D93" t="n">
-        <v>186.103019420931</v>
+        <v>186.1030042208767</v>
       </c>
       <c r="E93" t="n">
-        <v>186.8221435546875</v>
+        <v>186.8221282958984</v>
       </c>
       <c r="F93" t="n">
         <v>206188600</v>
@@ -2890,16 +2890,16 @@
         <v>46042</v>
       </c>
       <c r="B95" t="n">
-        <v>181.6783938022576</v>
+        <v>181.6784093892375</v>
       </c>
       <c r="C95" t="n">
-        <v>182.1578200140757</v>
+        <v>182.1578356421877</v>
       </c>
       <c r="D95" t="n">
-        <v>177.3936268105082</v>
+        <v>177.3936420298793</v>
       </c>
       <c r="E95" t="n">
-        <v>177.8530731201172</v>
+        <v>177.8530883789062</v>
       </c>
       <c r="F95" t="n">
         <v>223345300</v>
@@ -3046,16 +3046,16 @@
         <v>46050</v>
       </c>
       <c r="B101" t="n">
-        <v>191.0370019340606</v>
+        <v>191.0369866951896</v>
       </c>
       <c r="C101" t="n">
-        <v>192.1156881225865</v>
+        <v>192.1156727976695</v>
       </c>
       <c r="D101" t="n">
-        <v>189.6087360143659</v>
+        <v>189.6087208894265</v>
       </c>
       <c r="E101" t="n">
-        <v>191.2866973876953</v>
+        <v>191.2866821289062</v>
       </c>
       <c r="F101" t="n">
         <v>148552700</v>
@@ -3124,16 +3124,16 @@
         <v>46055</v>
       </c>
       <c r="B104" t="n">
-        <v>186.9719553243457</v>
+        <v>186.9719399348449</v>
       </c>
       <c r="C104" t="n">
-        <v>190.0681850900544</v>
+        <v>190.0681694457055</v>
       </c>
       <c r="D104" t="n">
-        <v>184.6547894061738</v>
+        <v>184.6547742073969</v>
       </c>
       <c r="E104" t="n">
-        <v>185.3838958740234</v>
+        <v>185.3838806152344</v>
       </c>
       <c r="F104" t="n">
         <v>165794100</v>
@@ -3176,16 +3176,16 @@
         <v>46057</v>
       </c>
       <c r="B106" t="n">
-        <v>179.2413826421603</v>
+        <v>179.241398362594</v>
       </c>
       <c r="C106" t="n">
-        <v>179.3612315773567</v>
+        <v>179.3612473083018</v>
       </c>
       <c r="D106" t="n">
-        <v>171.7005772519807</v>
+        <v>171.7005923110452</v>
       </c>
       <c r="E106" t="n">
-        <v>173.9777984619141</v>
+        <v>173.9778137207031</v>
       </c>
       <c r="F106" t="n">
         <v>207014100</v>
@@ -3202,16 +3202,16 @@
         <v>46058</v>
       </c>
       <c r="B107" t="n">
-        <v>174.7168806029182</v>
+        <v>174.7168961324724</v>
       </c>
       <c r="C107" t="n">
-        <v>176.604592702014</v>
+        <v>176.6046083993559</v>
       </c>
       <c r="D107" t="n">
-        <v>170.8216379544658</v>
+        <v>170.8216531377948</v>
       </c>
       <c r="E107" t="n">
-        <v>171.6706085205078</v>
+        <v>171.6706237792969</v>
       </c>
       <c r="F107" t="n">
         <v>206312900</v>
@@ -3228,16 +3228,16 @@
         <v>46059</v>
       </c>
       <c r="B108" t="n">
-        <v>176.4747497339287</v>
+        <v>176.4747642750831</v>
       </c>
       <c r="C108" t="n">
-        <v>186.7721871314613</v>
+        <v>186.7722025211031</v>
       </c>
       <c r="D108" t="n">
-        <v>174.3872995354016</v>
+        <v>174.3873139045544</v>
       </c>
       <c r="E108" t="n">
-        <v>185.1841278076172</v>
+        <v>185.1841430664062</v>
       </c>
       <c r="F108" t="n">
         <v>231346200</v>
@@ -3306,16 +3306,16 @@
         <v>46064</v>
       </c>
       <c r="B111" t="n">
-        <v>192.2155516352278</v>
+        <v>192.2155670867083</v>
       </c>
       <c r="C111" t="n">
-        <v>193.0245624433192</v>
+        <v>193.024577959833</v>
       </c>
       <c r="D111" t="n">
-        <v>188.5400419786642</v>
+        <v>188.5400571346844</v>
       </c>
       <c r="E111" t="n">
-        <v>189.8184814453125</v>
+        <v>189.8184967041016</v>
       </c>
       <c r="F111" t="n">
         <v>144192700</v>
@@ -3358,16 +3358,16 @@
         <v>46066</v>
       </c>
       <c r="B113" t="n">
-        <v>187.2516202842281</v>
+        <v>187.2516046356435</v>
       </c>
       <c r="C113" t="n">
-        <v>187.2716001888381</v>
+        <v>187.2715845385837</v>
       </c>
       <c r="D113" t="n">
-        <v>181.3687956932374</v>
+        <v>181.3687805362794</v>
       </c>
       <c r="E113" t="n">
-        <v>182.5873107910156</v>
+        <v>182.5872955322266</v>
       </c>
       <c r="F113" t="n">
         <v>161888000</v>
@@ -3488,16 +3488,16 @@
         <v>46076</v>
       </c>
       <c r="B118" t="n">
-        <v>191.1668392283931</v>
+        <v>191.1668239815537</v>
       </c>
       <c r="C118" t="n">
-        <v>193.7137359837344</v>
+        <v>193.7137205337629</v>
       </c>
       <c r="D118" t="n">
-        <v>189.3490641935772</v>
+        <v>189.3490490917175</v>
       </c>
       <c r="E118" t="n">
-        <v>191.3166656494141</v>
+        <v>191.316650390625</v>
       </c>
       <c r="F118" t="n">
         <v>171584800</v>
@@ -3696,16 +3696,16 @@
         <v>46086</v>
       </c>
       <c r="B126" t="n">
-        <v>180.9492987428603</v>
+        <v>180.9492836646731</v>
       </c>
       <c r="C126" t="n">
-        <v>183.8357775650134</v>
+        <v>183.835762246301</v>
       </c>
       <c r="D126" t="n">
-        <v>177.6633132926684</v>
+        <v>177.6632984882966</v>
       </c>
       <c r="E126" t="n">
-        <v>183.1166534423828</v>
+        <v>183.1166381835938</v>
       </c>
       <c r="F126" t="n">
         <v>198779700</v>
@@ -3722,16 +3722,16 @@
         <v>46087</v>
       </c>
       <c r="B127" t="n">
-        <v>179.6209064601764</v>
+        <v>179.6209218923013</v>
       </c>
       <c r="C127" t="n">
-        <v>182.5373473445644</v>
+        <v>182.5373630272553</v>
       </c>
       <c r="D127" t="n">
-        <v>176.6045965447985</v>
+        <v>176.6046117177772</v>
       </c>
       <c r="E127" t="n">
-        <v>177.6033782958984</v>
+        <v>177.6033935546875</v>
       </c>
       <c r="F127" t="n">
         <v>189021900</v>
@@ -3774,16 +3774,16 @@
         <v>46091</v>
       </c>
       <c r="B129" t="n">
-        <v>182.1777985889466</v>
+        <v>182.1777835258792</v>
       </c>
       <c r="C129" t="n">
-        <v>186.2128856921408</v>
+        <v>186.2128702954389</v>
       </c>
       <c r="D129" t="n">
-        <v>181.7882742872215</v>
+        <v>181.7882592563612</v>
       </c>
       <c r="E129" t="n">
-        <v>184.544921875</v>
+        <v>184.5449066162109</v>
       </c>
       <c r="F129" t="n">
         <v>179118500</v>
@@ -10937,7 +10937,7 @@
         <v>29.159492</v>
       </c>
       <c r="L2" t="n">
-        <v>14.902219</v>
+        <v>14.843682</v>
       </c>
       <c r="M2" t="n">
         <v>7.9</v>
@@ -11015,7 +11015,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:08:18</t>
+          <t>2026-09-08 08:52:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update NVDA data - 2026-09-12 21:48:06
</commit_message>
<xml_diff>
--- a/data/NVDA_data.xlsx
+++ b/data/NVDA_data.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H252"/>
+  <dimension ref="A1:H253"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,22 +433,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Open</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Close</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -471,20 +471,12 @@
       <c r="A2" s="1" t="n">
         <v>45911</v>
       </c>
-      <c r="B2" t="n">
-        <v>179.2505315119071</v>
-      </c>
-      <c r="C2" t="n">
-        <v>179.8491035140756</v>
-      </c>
-      <c r="D2" t="n">
-        <v>176.0581830190845</v>
-      </c>
-      <c r="E2" t="n">
-        <v>176.7465362548828</v>
-      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>151159300</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
         <v>0.01</v>
@@ -498,16 +490,16 @@
         <v>45912</v>
       </c>
       <c r="B3" t="n">
-        <v>177.3451359862166</v>
+        <v>177.3949890136719</v>
       </c>
       <c r="C3" t="n">
-        <v>178.1731541223449</v>
+        <v>178.1731234709029</v>
       </c>
       <c r="D3" t="n">
-        <v>176.028283464474</v>
+        <v>176.0282531820179</v>
       </c>
       <c r="E3" t="n">
-        <v>177.39501953125</v>
+        <v>177.34510547722</v>
       </c>
       <c r="F3" t="n">
         <v>124911000</v>
@@ -524,7 +516,7 @@
         <v>45915</v>
       </c>
       <c r="B4" t="n">
-        <v>175.2501343169162</v>
+        <v>177.3251647949219</v>
       </c>
       <c r="C4" t="n">
         <v>178.4225418052247</v>
@@ -533,7 +525,7 @@
         <v>174.0929031464731</v>
       </c>
       <c r="E4" t="n">
-        <v>177.3251647949219</v>
+        <v>175.2501343169162</v>
       </c>
       <c r="F4" t="n">
         <v>147061600</v>
@@ -550,7 +542,7 @@
         <v>45916</v>
       </c>
       <c r="B5" t="n">
-        <v>176.5769489507663</v>
+        <v>174.4620208740234</v>
       </c>
       <c r="C5" t="n">
         <v>177.0757538913052</v>
@@ -559,7 +551,7 @@
         <v>173.9632159334845</v>
       </c>
       <c r="E5" t="n">
-        <v>174.4620208740234</v>
+        <v>176.5769489507663</v>
       </c>
       <c r="F5" t="n">
         <v>140737800</v>
@@ -576,16 +568,16 @@
         <v>45917</v>
       </c>
       <c r="B6" t="n">
-        <v>172.2273696616015</v>
+        <v>169.8829956054688</v>
       </c>
       <c r="C6" t="n">
-        <v>172.7860287607356</v>
+        <v>172.7860442802747</v>
       </c>
       <c r="D6" t="n">
-        <v>168.007484117061</v>
+        <v>168.0074992073941</v>
       </c>
       <c r="E6" t="n">
-        <v>169.8829803466797</v>
+        <v>172.2273851309623</v>
       </c>
       <c r="F6" t="n">
         <v>211843800</v>
@@ -602,7 +594,7 @@
         <v>45918</v>
       </c>
       <c r="B7" t="n">
-        <v>173.5641783462465</v>
+        <v>175.8187866210938</v>
       </c>
       <c r="C7" t="n">
         <v>176.6767318043244</v>
@@ -611,7 +603,7 @@
         <v>172.5466271367534</v>
       </c>
       <c r="E7" t="n">
-        <v>175.8187866210938</v>
+        <v>173.5641783462465</v>
       </c>
       <c r="F7" t="n">
         <v>191763300</v>
@@ -628,7 +620,7 @@
         <v>45919</v>
       </c>
       <c r="B8" t="n">
-        <v>175.349898865447</v>
+        <v>176.2477416992188</v>
       </c>
       <c r="C8" t="n">
         <v>177.6543753314711</v>
@@ -637,7 +629,7 @@
         <v>174.7612974471592</v>
       </c>
       <c r="E8" t="n">
-        <v>176.2477416992188</v>
+        <v>175.349898865447</v>
       </c>
       <c r="F8" t="n">
         <v>237182100</v>
@@ -654,16 +646,16 @@
         <v>45922</v>
       </c>
       <c r="B9" t="n">
-        <v>174.8810364137678</v>
+        <v>183.1711578369141</v>
       </c>
       <c r="C9" t="n">
-        <v>184.1089289332547</v>
+        <v>184.1089135963474</v>
       </c>
       <c r="D9" t="n">
-        <v>174.2924501658818</v>
+        <v>174.2924356467209</v>
       </c>
       <c r="E9" t="n">
-        <v>183.1711730957031</v>
+        <v>174.8810218455756</v>
       </c>
       <c r="F9" t="n">
         <v>269637000</v>
@@ -680,7 +672,7 @@
         <v>45923</v>
       </c>
       <c r="B10" t="n">
-        <v>181.5350878652714</v>
+        <v>178.0035400390625</v>
       </c>
       <c r="C10" t="n">
         <v>181.9840093083128</v>
@@ -689,7 +681,7 @@
         <v>175.7888599052367</v>
       </c>
       <c r="E10" t="n">
-        <v>178.0035400390625</v>
+        <v>181.5350878652714</v>
       </c>
       <c r="F10" t="n">
         <v>192559600</v>
@@ -706,7 +698,7 @@
         <v>45924</v>
       </c>
       <c r="B11" t="n">
-        <v>179.3403383898065</v>
+        <v>176.5470275878906</v>
       </c>
       <c r="C11" t="n">
         <v>179.3503090089054</v>
@@ -715,7 +707,7 @@
         <v>174.9807727171775</v>
       </c>
       <c r="E11" t="n">
-        <v>176.5470275878906</v>
+        <v>179.3403383898065</v>
       </c>
       <c r="F11" t="n">
         <v>143564100</v>
@@ -732,7 +724,7 @@
         <v>45925</v>
       </c>
       <c r="B12" t="n">
-        <v>174.0629701066951</v>
+        <v>177.2653045654297</v>
       </c>
       <c r="C12" t="n">
         <v>179.8291540783439</v>
@@ -741,7 +733,7 @@
         <v>172.7162058826927</v>
       </c>
       <c r="E12" t="n">
-        <v>177.2653045654297</v>
+        <v>174.0629701066951</v>
       </c>
       <c r="F12" t="n">
         <v>191586700</v>
@@ -758,16 +750,16 @@
         <v>45926</v>
       </c>
       <c r="B13" t="n">
-        <v>177.7441426621237</v>
+        <v>177.7641143798828</v>
       </c>
       <c r="C13" t="n">
-        <v>179.3403244887289</v>
+        <v>179.3403398828169</v>
       </c>
       <c r="D13" t="n">
-        <v>174.5118813132914</v>
+        <v>174.5118962929188</v>
       </c>
       <c r="E13" t="n">
-        <v>177.7640991210938</v>
+        <v>177.7441579191998</v>
       </c>
       <c r="F13" t="n">
         <v>148573700</v>
@@ -784,7 +776,7 @@
         <v>45929</v>
       </c>
       <c r="B14" t="n">
-        <v>179.9987552370008</v>
+        <v>181.4153747558594</v>
       </c>
       <c r="C14" t="n">
         <v>183.5602300506758</v>
@@ -793,7 +785,7 @@
         <v>179.8890327563757</v>
       </c>
       <c r="E14" t="n">
-        <v>181.4153747558594</v>
+        <v>179.9987552370008</v>
       </c>
       <c r="F14" t="n">
         <v>193063500</v>
@@ -810,7 +802,7 @@
         <v>45930</v>
       </c>
       <c r="B15" t="n">
-        <v>181.6448190078555</v>
+        <v>186.1340637207031</v>
       </c>
       <c r="C15" t="n">
         <v>186.9022276338177</v>
@@ -819,7 +811,7 @@
         <v>181.0462469572146</v>
       </c>
       <c r="E15" t="n">
-        <v>186.1340637207031</v>
+        <v>181.6448190078555</v>
       </c>
       <c r="F15" t="n">
         <v>236981000</v>
@@ -836,7 +828,7 @@
         <v>45931</v>
       </c>
       <c r="B16" t="n">
-        <v>184.7972606974542</v>
+        <v>186.79248046875</v>
       </c>
       <c r="C16" t="n">
         <v>187.6903232769056</v>
@@ -845,7 +837,7 @@
         <v>183.4604518817237</v>
       </c>
       <c r="E16" t="n">
-        <v>186.79248046875</v>
+        <v>184.7972606974542</v>
       </c>
       <c r="F16" t="n">
         <v>173844900</v>
@@ -862,16 +854,16 @@
         <v>45932</v>
       </c>
       <c r="B17" t="n">
-        <v>189.146847340247</v>
+        <v>188.4385528564453</v>
       </c>
       <c r="C17" t="n">
-        <v>190.59337868299</v>
+        <v>190.593394116267</v>
       </c>
       <c r="D17" t="n">
-        <v>187.6105195355423</v>
+        <v>187.6105347272827</v>
       </c>
       <c r="E17" t="n">
-        <v>188.4385375976562</v>
+        <v>189.1468626563914</v>
       </c>
       <c r="F17" t="n">
         <v>136805800</v>
@@ -888,16 +880,16 @@
         <v>45933</v>
       </c>
       <c r="B18" t="n">
-        <v>188.7378247179256</v>
+        <v>187.1715545654297</v>
       </c>
       <c r="C18" t="n">
-        <v>189.9050265070322</v>
+        <v>189.9050110254035</v>
       </c>
       <c r="D18" t="n">
-        <v>184.9369333277354</v>
+        <v>184.9369182511207</v>
       </c>
       <c r="E18" t="n">
-        <v>187.1715698242188</v>
+        <v>188.7378093314507</v>
       </c>
       <c r="F18" t="n">
         <v>137596900</v>
@@ -914,16 +906,16 @@
         <v>45936</v>
       </c>
       <c r="B19" t="n">
-        <v>185.0566599139491</v>
+        <v>185.0965423583984</v>
       </c>
       <c r="C19" t="n">
-        <v>186.7825209975275</v>
+        <v>186.7825055997528</v>
       </c>
       <c r="D19" t="n">
-        <v>182.8918479831437</v>
+        <v>182.8918329061041</v>
       </c>
       <c r="E19" t="n">
-        <v>185.0965576171875</v>
+        <v>185.0566446584491</v>
       </c>
       <c r="F19" t="n">
         <v>157678100</v>
@@ -940,16 +932,16 @@
         <v>45937</v>
       </c>
       <c r="B20" t="n">
-        <v>185.784875425114</v>
+        <v>184.5977325439453</v>
       </c>
       <c r="C20" t="n">
-        <v>188.6081130865945</v>
+        <v>188.6081286768816</v>
       </c>
       <c r="D20" t="n">
-        <v>183.5602097539322</v>
+        <v>183.5602249269612</v>
       </c>
       <c r="E20" t="n">
-        <v>184.5977172851562</v>
+        <v>185.7848907820332</v>
       </c>
       <c r="F20" t="n">
         <v>140088000</v>
@@ -966,16 +958,16 @@
         <v>45938</v>
       </c>
       <c r="B21" t="n">
-        <v>186.1240974206304</v>
+        <v>188.6580047607422</v>
       </c>
       <c r="C21" t="n">
-        <v>189.1468543796426</v>
+        <v>189.1468390813163</v>
       </c>
       <c r="D21" t="n">
-        <v>186.0941551173159</v>
+        <v>186.094140065894</v>
       </c>
       <c r="E21" t="n">
-        <v>188.6580200195312</v>
+        <v>186.1240823667868</v>
       </c>
       <c r="F21" t="n">
         <v>130168900</v>
@@ -992,7 +984,7 @@
         <v>45939</v>
       </c>
       <c r="B22" t="n">
-        <v>191.7705422839889</v>
+        <v>192.1097412109375</v>
       </c>
       <c r="C22" t="n">
         <v>194.8332119113436</v>
@@ -1001,7 +993,7 @@
         <v>190.6033405552435</v>
       </c>
       <c r="E22" t="n">
-        <v>192.1097412109375</v>
+        <v>191.7705422839889</v>
       </c>
       <c r="F22" t="n">
         <v>182997200</v>
@@ -1018,7 +1010,7 @@
         <v>45940</v>
       </c>
       <c r="B23" t="n">
-        <v>193.0474821132437</v>
+        <v>182.7222290039062</v>
       </c>
       <c r="C23" t="n">
         <v>195.1524395658232</v>
@@ -1027,7 +1019,7 @@
         <v>181.6148814298513</v>
       </c>
       <c r="E23" t="n">
-        <v>182.7222290039062</v>
+        <v>193.0474821132437</v>
       </c>
       <c r="F23" t="n">
         <v>268774400</v>
@@ -1044,16 +1036,16 @@
         <v>45943</v>
       </c>
       <c r="B24" t="n">
-        <v>187.52074924116</v>
+        <v>187.8699035644531</v>
       </c>
       <c r="C24" t="n">
-        <v>189.6556339904095</v>
+        <v>189.6556185865847</v>
       </c>
       <c r="D24" t="n">
-        <v>185.5155586605101</v>
+        <v>185.5155435929421</v>
       </c>
       <c r="E24" t="n">
-        <v>187.8699188232422</v>
+        <v>187.5207340107304</v>
       </c>
       <c r="F24" t="n">
         <v>153482800</v>
@@ -1070,7 +1062,7 @@
         <v>45944</v>
       </c>
       <c r="B25" t="n">
-        <v>184.3283927796865</v>
+        <v>179.5997161865234</v>
       </c>
       <c r="C25" t="n">
         <v>184.3583198600852</v>
@@ -1079,7 +1071,7 @@
         <v>179.2705030798172</v>
       </c>
       <c r="E25" t="n">
-        <v>179.5997161865234</v>
+        <v>184.3283927796865</v>
       </c>
       <c r="F25" t="n">
         <v>205641400</v>
@@ -1096,16 +1088,16 @@
         <v>45945</v>
       </c>
       <c r="B26" t="n">
-        <v>184.3582990595379</v>
+        <v>179.4001922607422</v>
       </c>
       <c r="C26" t="n">
-        <v>184.4281238318171</v>
+        <v>184.4281395182556</v>
       </c>
       <c r="D26" t="n">
-        <v>176.8662395170747</v>
+        <v>176.866254560341</v>
       </c>
       <c r="E26" t="n">
-        <v>179.4001770019531</v>
+        <v>184.3583147400375</v>
       </c>
       <c r="F26" t="n">
         <v>214450500</v>
@@ -1122,7 +1114,7 @@
         <v>45946</v>
       </c>
       <c r="B27" t="n">
-        <v>181.7944521048813</v>
+        <v>181.3754577636719</v>
       </c>
       <c r="C27" t="n">
         <v>182.8419455690647</v>
@@ -1131,7 +1123,7 @@
         <v>179.3403402174659</v>
       </c>
       <c r="E27" t="n">
-        <v>181.3754577636719</v>
+        <v>181.7944521048813</v>
       </c>
       <c r="F27" t="n">
         <v>179723300</v>
@@ -1148,16 +1140,16 @@
         <v>45947</v>
       </c>
       <c r="B28" t="n">
-        <v>179.7493465774322</v>
+        <v>182.7821044921875</v>
       </c>
       <c r="C28" t="n">
-        <v>183.6599908268075</v>
+        <v>183.6600061588844</v>
       </c>
       <c r="D28" t="n">
-        <v>179.3203816221287</v>
+        <v>179.3203965919317</v>
       </c>
       <c r="E28" t="n">
-        <v>182.7820892333984</v>
+        <v>179.7493615830456</v>
       </c>
       <c r="F28" t="n">
         <v>173135200</v>
@@ -1174,7 +1166,7 @@
         <v>45950</v>
       </c>
       <c r="B29" t="n">
-        <v>182.6923102950553</v>
+        <v>182.2034759521484</v>
       </c>
       <c r="C29" t="n">
         <v>184.7573549226016</v>
@@ -1183,7 +1175,7 @@
         <v>181.2956472677441</v>
       </c>
       <c r="E29" t="n">
-        <v>182.2034759521484</v>
+        <v>182.6923102950553</v>
       </c>
       <c r="F29" t="n">
         <v>128544700</v>
@@ -1200,7 +1192,7 @@
         <v>45951</v>
       </c>
       <c r="B30" t="n">
-        <v>182.3531141136141</v>
+        <v>180.7270202636719</v>
       </c>
       <c r="C30" t="n">
         <v>182.3531141136141</v>
@@ -1209,7 +1201,7 @@
         <v>179.3702701372806</v>
       </c>
       <c r="E30" t="n">
-        <v>180.7270202636719</v>
+        <v>182.3531141136141</v>
       </c>
       <c r="F30" t="n">
         <v>124240200</v>
@@ -1226,16 +1218,16 @@
         <v>45952</v>
       </c>
       <c r="B31" t="n">
-        <v>180.7070662621498</v>
+        <v>179.8491058349609</v>
       </c>
       <c r="C31" t="n">
-        <v>183.0015721983185</v>
+        <v>183.0015566720687</v>
       </c>
       <c r="D31" t="n">
-        <v>176.3375297972393</v>
+        <v>176.3375148363812</v>
       </c>
       <c r="E31" t="n">
-        <v>179.84912109375</v>
+        <v>180.7070509305708</v>
       </c>
       <c r="F31" t="n">
         <v>162249600</v>
@@ -1252,16 +1244,16 @@
         <v>45953</v>
       </c>
       <c r="B32" t="n">
-        <v>179.988777912505</v>
+        <v>181.7246398925781</v>
       </c>
       <c r="C32" t="n">
-        <v>182.5925403832715</v>
+        <v>182.5925557149365</v>
       </c>
       <c r="D32" t="n">
-        <v>179.3602787988416</v>
+        <v>179.3602938591047</v>
       </c>
       <c r="E32" t="n">
-        <v>181.7246246337891</v>
+        <v>179.988793025541</v>
       </c>
       <c r="F32" t="n">
         <v>111363700</v>
@@ -1278,16 +1270,16 @@
         <v>45954</v>
       </c>
       <c r="B33" t="n">
-        <v>183.4006051417061</v>
+        <v>185.8148040771484</v>
       </c>
       <c r="C33" t="n">
-        <v>187.0219340442129</v>
+        <v>187.0219186862977</v>
       </c>
       <c r="D33" t="n">
-        <v>183.0614214202242</v>
+        <v>183.0614063875393</v>
       </c>
       <c r="E33" t="n">
-        <v>185.8148193359375</v>
+        <v>183.400590081168</v>
       </c>
       <c r="F33" t="n">
         <v>131296700</v>
@@ -1304,7 +1296,7 @@
         <v>45957</v>
       </c>
       <c r="B34" t="n">
-        <v>189.5359184602369</v>
+        <v>191.0323333740234</v>
       </c>
       <c r="C34" t="n">
         <v>191.5411089646758</v>
@@ -1313,7 +1305,7 @@
         <v>187.9796341631504</v>
       </c>
       <c r="E34" t="n">
-        <v>191.0323333740234</v>
+        <v>189.5359184602369</v>
       </c>
       <c r="F34" t="n">
         <v>153452700</v>
@@ -1330,16 +1322,16 @@
         <v>45958</v>
       </c>
       <c r="B35" t="n">
-        <v>192.588592118433</v>
+        <v>200.5495300292969</v>
       </c>
       <c r="C35" t="n">
-        <v>202.6644428640734</v>
+        <v>202.6644582837766</v>
       </c>
       <c r="D35" t="n">
-        <v>191.4513174538508</v>
+        <v>191.4513320204045</v>
       </c>
       <c r="E35" t="n">
-        <v>200.5495147705078</v>
+        <v>192.5886067715161</v>
       </c>
       <c r="F35" t="n">
         <v>297986200</v>
@@ -1356,16 +1348,16 @@
         <v>45959</v>
       </c>
       <c r="B36" t="n">
-        <v>207.482906515472</v>
+        <v>206.545166015625</v>
       </c>
       <c r="C36" t="n">
-        <v>211.6828509687219</v>
+        <v>211.6828666070652</v>
       </c>
       <c r="D36" t="n">
-        <v>204.2905578218423</v>
+        <v>204.2905729140704</v>
       </c>
       <c r="E36" t="n">
-        <v>206.5451507568359</v>
+        <v>207.482921843539</v>
       </c>
       <c r="F36" t="n">
         <v>308829600</v>
@@ -1382,16 +1374,16 @@
         <v>45960</v>
       </c>
       <c r="B37" t="n">
-        <v>204.6596525726598</v>
+        <v>202.4050750732422</v>
       </c>
       <c r="C37" t="n">
-        <v>205.6672482532724</v>
+        <v>205.6672637579894</v>
       </c>
       <c r="D37" t="n">
-        <v>200.9286015136062</v>
+        <v>200.9286166610889</v>
       </c>
       <c r="E37" t="n">
-        <v>202.4050598144531</v>
+        <v>204.6596680014167</v>
       </c>
       <c r="F37" t="n">
         <v>178864400</v>
@@ -1408,16 +1400,16 @@
         <v>45961</v>
       </c>
       <c r="B38" t="n">
-        <v>205.9565693232556</v>
+        <v>202.0060272216797</v>
       </c>
       <c r="C38" t="n">
-        <v>207.4729406961805</v>
+        <v>207.4729250244422</v>
       </c>
       <c r="D38" t="n">
-        <v>201.5870481318289</v>
+        <v>201.5870329046891</v>
       </c>
       <c r="E38" t="n">
-        <v>202.0060424804688</v>
+        <v>205.9565537660584</v>
       </c>
       <c r="F38" t="n">
         <v>179802200</v>
@@ -1434,7 +1426,7 @@
         <v>45964</v>
       </c>
       <c r="B39" t="n">
-        <v>207.5826726752522</v>
+        <v>206.3855438232422</v>
       </c>
       <c r="C39" t="n">
         <v>210.8348755139714</v>
@@ -1443,7 +1435,7 @@
         <v>205.0686914304077</v>
       </c>
       <c r="E39" t="n">
-        <v>206.3855438232422</v>
+        <v>207.5826726752522</v>
       </c>
       <c r="F39" t="n">
         <v>180267300</v>
@@ -1460,7 +1452,7 @@
         <v>45965</v>
       </c>
       <c r="B40" t="n">
-        <v>202.5148147488263</v>
+        <v>198.2151184082031</v>
       </c>
       <c r="C40" t="n">
         <v>203.4824975937368</v>
@@ -1469,7 +1461,7 @@
         <v>197.4569251230167</v>
       </c>
       <c r="E40" t="n">
-        <v>198.2151184082031</v>
+        <v>202.5148147488263</v>
       </c>
       <c r="F40" t="n">
         <v>188919300</v>
@@ -1486,16 +1478,16 @@
         <v>45966</v>
       </c>
       <c r="B41" t="n">
-        <v>198.2949120548774</v>
+        <v>194.7434387207031</v>
       </c>
       <c r="C41" t="n">
-        <v>202.4349867997753</v>
+        <v>202.4350026612236</v>
       </c>
       <c r="D41" t="n">
-        <v>194.1847491650603</v>
+        <v>194.1847643800754</v>
       </c>
       <c r="E41" t="n">
-        <v>194.7434234619141</v>
+        <v>198.2949275919373</v>
       </c>
       <c r="F41" t="n">
         <v>171350300</v>
@@ -1512,7 +1504,7 @@
         <v>45967</v>
       </c>
       <c r="B42" t="n">
-        <v>195.9505410878136</v>
+        <v>187.6304779052734</v>
       </c>
       <c r="C42" t="n">
         <v>197.1476699621838</v>
@@ -1521,7 +1513,7 @@
         <v>185.9345440647224</v>
       </c>
       <c r="E42" t="n">
-        <v>187.6304779052734</v>
+        <v>195.9505410878136</v>
       </c>
       <c r="F42" t="n">
         <v>223029800</v>
@@ -1538,16 +1530,16 @@
         <v>45968</v>
       </c>
       <c r="B43" t="n">
-        <v>184.4580548583195</v>
+        <v>187.7003021240234</v>
       </c>
       <c r="C43" t="n">
-        <v>187.8698939350823</v>
+        <v>187.8699092076593</v>
       </c>
       <c r="D43" t="n">
-        <v>178.4823816093971</v>
+        <v>178.4823961188316</v>
       </c>
       <c r="E43" t="n">
-        <v>187.7002868652344</v>
+        <v>184.4580698535366</v>
       </c>
       <c r="F43" t="n">
         <v>264942300</v>
@@ -1564,16 +1556,16 @@
         <v>45971</v>
       </c>
       <c r="B44" t="n">
-        <v>194.6436639125443</v>
+        <v>198.5742645263672</v>
       </c>
       <c r="C44" t="n">
-        <v>199.4621214501376</v>
+        <v>199.4621367771523</v>
       </c>
       <c r="D44" t="n">
-        <v>193.3268115668235</v>
+        <v>193.3268264223904</v>
       </c>
       <c r="E44" t="n">
-        <v>198.5742492675781</v>
+        <v>194.6436788693004</v>
       </c>
       <c r="F44" t="n">
         <v>198897100</v>
@@ -1590,7 +1582,7 @@
         <v>45972</v>
       </c>
       <c r="B45" t="n">
-        <v>194.6935535589016</v>
+        <v>192.6983337402344</v>
       </c>
       <c r="C45" t="n">
         <v>194.9529266552934</v>
@@ -1599,7 +1591,7 @@
         <v>190.8427786999811</v>
       </c>
       <c r="E45" t="n">
-        <v>192.6983337402344</v>
+        <v>194.6935535589016</v>
       </c>
       <c r="F45" t="n">
         <v>176483300</v>
@@ -1616,16 +1608,16 @@
         <v>45973</v>
       </c>
       <c r="B46" t="n">
-        <v>195.2522010776849</v>
+        <v>193.3368072509766</v>
       </c>
       <c r="C46" t="n">
-        <v>195.4217929255223</v>
+        <v>195.4218083488666</v>
       </c>
       <c r="D46" t="n">
-        <v>190.6731755191215</v>
+        <v>190.673190567689</v>
       </c>
       <c r="E46" t="n">
-        <v>193.3367919921875</v>
+        <v>195.2522164876445</v>
       </c>
       <c r="F46" t="n">
         <v>154935300</v>
@@ -1642,16 +1634,16 @@
         <v>45974</v>
       </c>
       <c r="B47" t="n">
-        <v>190.5933791327836</v>
+        <v>186.4133758544922</v>
       </c>
       <c r="C47" t="n">
-        <v>190.9824463944715</v>
+        <v>190.9824307616844</v>
       </c>
       <c r="D47" t="n">
-        <v>183.4105907203728</v>
+        <v>183.4105757073767</v>
       </c>
       <c r="E47" t="n">
-        <v>186.4133911132812</v>
+        <v>190.5933635318434</v>
       </c>
       <c r="F47" t="n">
         <v>207423100</v>
@@ -1668,7 +1660,7 @@
         <v>45975</v>
       </c>
       <c r="B48" t="n">
-        <v>182.4229435613052</v>
+        <v>189.7154693603516</v>
       </c>
       <c r="C48" t="n">
         <v>190.553458007553</v>
@@ -1677,7 +1669,7 @@
         <v>180.1483942490048</v>
       </c>
       <c r="E48" t="n">
-        <v>189.7154693603516</v>
+        <v>182.4229435613052</v>
       </c>
       <c r="F48" t="n">
         <v>186591900</v>
@@ -1694,16 +1686,16 @@
         <v>45978</v>
       </c>
       <c r="B49" t="n">
-        <v>185.5255230789849</v>
+        <v>186.1540069580078</v>
       </c>
       <c r="C49" t="n">
-        <v>188.5482800008962</v>
+        <v>188.5482645458532</v>
       </c>
       <c r="D49" t="n">
-        <v>183.8794727552066</v>
+        <v>183.8794576828592</v>
       </c>
       <c r="E49" t="n">
-        <v>186.1540222167969</v>
+        <v>185.525507871713</v>
       </c>
       <c r="F49" t="n">
         <v>173628900</v>
@@ -1720,16 +1712,16 @@
         <v>45979</v>
       </c>
       <c r="B50" t="n">
-        <v>182.9417205846578</v>
+        <v>180.926513671875</v>
       </c>
       <c r="C50" t="n">
-        <v>184.3583249108488</v>
+        <v>184.358293814419</v>
       </c>
       <c r="D50" t="n">
-        <v>179.2206244483882</v>
+        <v>179.2205942185541</v>
       </c>
       <c r="E50" t="n">
-        <v>180.9265441894531</v>
+        <v>182.9416897271721</v>
       </c>
       <c r="F50" t="n">
         <v>213598900</v>
@@ -1746,16 +1738,16 @@
         <v>45980</v>
       </c>
       <c r="B51" t="n">
-        <v>184.3483273978252</v>
+        <v>186.0741882324219</v>
       </c>
       <c r="C51" t="n">
-        <v>187.4109971087465</v>
+        <v>187.4109817403353</v>
       </c>
       <c r="D51" t="n">
-        <v>182.3930205111681</v>
+        <v>182.39300555425</v>
       </c>
       <c r="E51" t="n">
-        <v>186.0742034912109</v>
+        <v>184.3483122805645</v>
       </c>
       <c r="F51" t="n">
         <v>247246400</v>
@@ -1772,16 +1764,16 @@
         <v>45981</v>
       </c>
       <c r="B52" t="n">
-        <v>195.4816405536745</v>
+        <v>180.208251953125</v>
       </c>
       <c r="C52" t="n">
-        <v>195.5315240889771</v>
+        <v>195.5315406452363</v>
       </c>
       <c r="D52" t="n">
-        <v>179.4201316368992</v>
+        <v>179.4201468289569</v>
       </c>
       <c r="E52" t="n">
-        <v>180.2082366943359</v>
+        <v>195.4816571057099</v>
       </c>
       <c r="F52" t="n">
         <v>343504800</v>
@@ -1798,16 +1790,16 @@
         <v>45982</v>
       </c>
       <c r="B53" t="n">
-        <v>180.8068289121023</v>
+        <v>178.4524536132812</v>
       </c>
       <c r="C53" t="n">
-        <v>184.1188859589464</v>
+        <v>184.1188702156436</v>
       </c>
       <c r="D53" t="n">
-        <v>172.5166776199441</v>
+        <v>172.5166628687019</v>
       </c>
       <c r="E53" t="n">
-        <v>178.4524688720703</v>
+        <v>180.806813452001</v>
       </c>
       <c r="F53" t="n">
         <v>346926200</v>
@@ -1824,16 +1816,16 @@
         <v>45985</v>
       </c>
       <c r="B54" t="n">
-        <v>179.0610243324759</v>
+        <v>182.1136932373047</v>
       </c>
       <c r="C54" t="n">
-        <v>183.0614349513779</v>
+        <v>183.0614196131816</v>
       </c>
       <c r="D54" t="n">
-        <v>176.0582084909882</v>
+        <v>176.0581937395723</v>
       </c>
       <c r="E54" t="n">
-        <v>182.1137084960938</v>
+        <v>179.0610093294625</v>
       </c>
       <c r="F54" t="n">
         <v>256618300</v>
@@ -1850,16 +1842,16 @@
         <v>45986</v>
       </c>
       <c r="B55" t="n">
-        <v>174.4919707447618</v>
+        <v>177.3949890136719</v>
       </c>
       <c r="C55" t="n">
-        <v>177.734203281764</v>
+        <v>177.7341727058355</v>
       </c>
       <c r="D55" t="n">
-        <v>169.1447804748437</v>
+        <v>169.1447513765687</v>
       </c>
       <c r="E55" t="n">
-        <v>177.39501953125</v>
+        <v>174.4919407266003</v>
       </c>
       <c r="F55" t="n">
         <v>320600300</v>
@@ -1876,7 +1868,7 @@
         <v>45987</v>
       </c>
       <c r="B56" t="n">
-        <v>181.1958831941039</v>
+        <v>179.8291473388672</v>
       </c>
       <c r="C56" t="n">
         <v>182.4728225932506</v>
@@ -1885,7 +1877,7 @@
         <v>177.8139863878403</v>
       </c>
       <c r="E56" t="n">
-        <v>179.8291473388672</v>
+        <v>181.1958831941039</v>
       </c>
       <c r="F56" t="n">
         <v>183852000</v>
@@ -1902,16 +1894,16 @@
         <v>45989</v>
       </c>
       <c r="B57" t="n">
-        <v>178.5821558989869</v>
+        <v>176.5769500732422</v>
       </c>
       <c r="C57" t="n">
-        <v>178.8614854738169</v>
+        <v>178.8614700176124</v>
       </c>
       <c r="D57" t="n">
-        <v>176.0781603452176</v>
+        <v>176.0781451295325</v>
       </c>
       <c r="E57" t="n">
-        <v>176.5769653320312</v>
+        <v>178.5821404669205</v>
       </c>
       <c r="F57" t="n">
         <v>121332800</v>
@@ -1928,16 +1920,16 @@
         <v>45992</v>
       </c>
       <c r="B58" t="n">
-        <v>174.3423041351479</v>
+        <v>179.489990234375</v>
       </c>
       <c r="C58" t="n">
-        <v>179.8690716163194</v>
+        <v>179.8690869073362</v>
       </c>
       <c r="D58" t="n">
-        <v>173.2648835948944</v>
+        <v>173.2648983244765</v>
       </c>
       <c r="E58" t="n">
-        <v>179.4899749755859</v>
+        <v>174.3423189563235</v>
       </c>
       <c r="F58" t="n">
         <v>188131000</v>
@@ -1954,7 +1946,7 @@
         <v>45993</v>
       </c>
       <c r="B59" t="n">
-        <v>181.3255769560617</v>
+        <v>181.0263061523438</v>
       </c>
       <c r="C59" t="n">
         <v>185.2162648499111</v>
@@ -1963,7 +1955,7 @@
         <v>179.569788944198</v>
       </c>
       <c r="E59" t="n">
-        <v>181.0263061523438</v>
+        <v>181.3255769560617</v>
       </c>
       <c r="F59" t="n">
         <v>182632200</v>
@@ -1980,7 +1972,7 @@
         <v>45994</v>
       </c>
       <c r="B60" t="n">
-        <v>180.6472109015755</v>
+        <v>179.1607666015625</v>
       </c>
       <c r="C60" t="n">
         <v>182.0139316568558</v>
@@ -1989,7 +1981,7 @@
         <v>178.681918089591</v>
       </c>
       <c r="E60" t="n">
-        <v>179.1607666015625</v>
+        <v>180.6472109015755</v>
       </c>
       <c r="F60" t="n">
         <v>165138000</v>
@@ -2006,7 +1998,7 @@
         <v>45995</v>
       </c>
       <c r="B61" t="n">
-        <v>181.1959881613664</v>
+        <v>182.9518890380859</v>
       </c>
       <c r="C61" t="n">
         <v>184.089227004522</v>
@@ -2015,7 +2007,7 @@
         <v>179.5398751387779</v>
       </c>
       <c r="E61" t="n">
-        <v>182.9518890380859</v>
+        <v>181.1959881613664</v>
       </c>
       <c r="F61" t="n">
         <v>167364900</v>
@@ -2032,7 +2024,7 @@
         <v>45996</v>
       </c>
       <c r="B62" t="n">
-        <v>183.4607020047171</v>
+        <v>181.9841613769531</v>
       </c>
       <c r="C62" t="n">
         <v>184.2289086763207</v>
@@ -2041,7 +2033,7 @@
         <v>180.4876631773748</v>
       </c>
       <c r="E62" t="n">
-        <v>181.9841613769531</v>
+        <v>183.4607020047171</v>
       </c>
       <c r="F62" t="n">
         <v>143971100</v>
@@ -2058,16 +2050,16 @@
         <v>45999</v>
       </c>
       <c r="B63" t="n">
-        <v>182.213626289633</v>
+        <v>185.1168212890625</v>
       </c>
       <c r="C63" t="n">
-        <v>187.5611139779305</v>
+        <v>187.5610985176648</v>
       </c>
       <c r="D63" t="n">
-        <v>181.9741810893209</v>
+        <v>181.9741660895743</v>
       </c>
       <c r="E63" t="n">
-        <v>185.1168365478516</v>
+        <v>182.2136112701494</v>
       </c>
       <c r="F63" t="n">
         <v>204378100</v>
@@ -2084,16 +2076,16 @@
         <v>46000</v>
       </c>
       <c r="B64" t="n">
-        <v>185.12679644575</v>
+        <v>184.5381927490234</v>
       </c>
       <c r="C64" t="n">
-        <v>185.2864265695677</v>
+        <v>185.2864418902268</v>
       </c>
       <c r="D64" t="n">
-        <v>182.8920356049676</v>
+        <v>182.8920507276432</v>
       </c>
       <c r="E64" t="n">
-        <v>184.5381774902344</v>
+        <v>185.1268117532098</v>
       </c>
       <c r="F64" t="n">
         <v>144719700</v>
@@ -2110,16 +2102,16 @@
         <v>46001</v>
       </c>
       <c r="B65" t="n">
-        <v>184.5381918075859</v>
+        <v>183.3509521484375</v>
       </c>
       <c r="C65" t="n">
-        <v>185.0469957406681</v>
+        <v>185.0469803407326</v>
       </c>
       <c r="D65" t="n">
-        <v>181.6150239281505</v>
+        <v>181.6150088138297</v>
       </c>
       <c r="E65" t="n">
-        <v>183.3509674072266</v>
+        <v>184.538176449994</v>
       </c>
       <c r="F65" t="n">
         <v>162785400</v>
@@ -2136,7 +2128,7 @@
         <v>46002</v>
       </c>
       <c r="B66" t="n">
-        <v>179.8591224369562</v>
+        <v>180.5075988769531</v>
       </c>
       <c r="C66" t="n">
         <v>180.8967030087509</v>
@@ -2145,7 +2137,7 @@
         <v>176.2076633109278</v>
       </c>
       <c r="E66" t="n">
-        <v>180.5075988769531</v>
+        <v>179.8591224369562</v>
       </c>
       <c r="F66" t="n">
         <v>182136600</v>
@@ -2162,16 +2154,16 @@
         <v>46003</v>
       </c>
       <c r="B67" t="n">
-        <v>180.6871831157045</v>
+        <v>174.6114196777344</v>
       </c>
       <c r="C67" t="n">
-        <v>182.3931976659576</v>
+        <v>182.3932136047752</v>
       </c>
       <c r="D67" t="n">
-        <v>174.2123291208211</v>
+        <v>174.2123443447362</v>
       </c>
       <c r="E67" t="n">
-        <v>174.6114044189453</v>
+        <v>180.6871989054384</v>
       </c>
       <c r="F67" t="n">
         <v>204274900</v>
@@ -2188,16 +2180,16 @@
         <v>46006</v>
       </c>
       <c r="B68" t="n">
-        <v>177.5245749312296</v>
+        <v>175.8784332275391</v>
       </c>
       <c r="C68" t="n">
-        <v>178.0034500370577</v>
+        <v>178.0034654802094</v>
       </c>
       <c r="D68" t="n">
-        <v>174.6213651072644</v>
+        <v>174.6213802569945</v>
       </c>
       <c r="E68" t="n">
-        <v>175.87841796875</v>
+        <v>177.5245903328353</v>
       </c>
       <c r="F68" t="n">
         <v>164775600</v>
@@ -2214,7 +2206,7 @@
         <v>46007</v>
       </c>
       <c r="B69" t="n">
-        <v>175.8485012773324</v>
+        <v>177.3050994873047</v>
       </c>
       <c r="C69" t="n">
         <v>178.0733061224419</v>
@@ -2223,7 +2215,7 @@
         <v>174.4916756985292</v>
       </c>
       <c r="E69" t="n">
-        <v>177.3050994873047</v>
+        <v>175.8485012773324</v>
       </c>
       <c r="F69" t="n">
         <v>148588100</v>
@@ -2240,16 +2232,16 @@
         <v>46008</v>
       </c>
       <c r="B70" t="n">
-        <v>175.6888811343</v>
+        <v>170.5409393310547</v>
       </c>
       <c r="C70" t="n">
-        <v>175.7188098781239</v>
+        <v>175.7188256001934</v>
       </c>
       <c r="D70" t="n">
-        <v>169.9123900056319</v>
+        <v>169.9124052081842</v>
       </c>
       <c r="E70" t="n">
-        <v>170.5409240722656</v>
+        <v>175.6888968536916</v>
       </c>
       <c r="F70" t="n">
         <v>222775500</v>
@@ -2266,7 +2258,7 @@
         <v>46009</v>
       </c>
       <c r="B71" t="n">
-        <v>174.1225483861358</v>
+        <v>173.7334594726562</v>
       </c>
       <c r="C71" t="n">
         <v>175.7387615308714</v>
@@ -2275,7 +2267,7 @@
         <v>171.4188835631069</v>
       </c>
       <c r="E71" t="n">
-        <v>173.7334594726562</v>
+        <v>174.1225483861358</v>
       </c>
       <c r="F71" t="n">
         <v>176096000</v>
@@ -2292,16 +2284,16 @@
         <v>46010</v>
       </c>
       <c r="B72" t="n">
-        <v>176.2575672304301</v>
+        <v>180.5674743652344</v>
       </c>
       <c r="C72" t="n">
-        <v>181.0264072425164</v>
+        <v>181.0263919449467</v>
       </c>
       <c r="D72" t="n">
-        <v>175.9283357789888</v>
+        <v>175.9283209122297</v>
       </c>
       <c r="E72" t="n">
-        <v>180.5674896240234</v>
+        <v>176.2575523358494</v>
       </c>
       <c r="F72" t="n">
         <v>324925900</v>
@@ -2318,7 +2310,7 @@
         <v>46013</v>
       </c>
       <c r="B73" t="n">
-        <v>183.4906282252173</v>
+        <v>183.2611694335938</v>
       </c>
       <c r="C73" t="n">
         <v>183.7300734141942</v>
@@ -2327,7 +2319,7 @@
         <v>181.9243013805983</v>
       </c>
       <c r="E73" t="n">
-        <v>183.2611694335938</v>
+        <v>183.4906282252173</v>
       </c>
       <c r="F73" t="n">
         <v>129064400</v>
@@ -2344,7 +2336,7 @@
         <v>46014</v>
       </c>
       <c r="B74" t="n">
-        <v>182.5428571096804</v>
+        <v>188.7682952880859</v>
       </c>
       <c r="C74" t="n">
         <v>188.8880102762506</v>
@@ -2353,7 +2345,7 @@
         <v>182.4730132178061</v>
       </c>
       <c r="E74" t="n">
-        <v>188.7682952880859</v>
+        <v>182.5428571096804</v>
       </c>
       <c r="F74" t="n">
         <v>174873600</v>
@@ -2370,7 +2362,7 @@
         <v>46015</v>
       </c>
       <c r="B75" t="n">
-        <v>187.5012437217294</v>
+        <v>188.169677734375</v>
       </c>
       <c r="C75" t="n">
         <v>188.4689804086018</v>
@@ -2379,7 +2371,7 @@
         <v>186.154389299292</v>
       </c>
       <c r="E75" t="n">
-        <v>188.169677734375</v>
+        <v>187.5012437217294</v>
       </c>
       <c r="F75" t="n">
         <v>65528500</v>
@@ -2396,7 +2388,7 @@
         <v>46017</v>
       </c>
       <c r="B76" t="n">
-        <v>189.4766285187414</v>
+        <v>190.085205078125</v>
       </c>
       <c r="C76" t="n">
         <v>192.240166195598</v>
@@ -2405,7 +2397,7 @@
         <v>187.5611125998212</v>
       </c>
       <c r="E76" t="n">
-        <v>190.085205078125</v>
+        <v>189.4766285187414</v>
       </c>
       <c r="F76" t="n">
         <v>139740300</v>
@@ -2422,7 +2414,7 @@
         <v>46020</v>
       </c>
       <c r="B77" t="n">
-        <v>187.2717899684254</v>
+        <v>187.7805938720703</v>
       </c>
       <c r="C77" t="n">
         <v>188.3193265216257</v>
@@ -2431,7 +2423,7 @@
         <v>185.4759890979627</v>
       </c>
       <c r="E77" t="n">
-        <v>187.7805938720703</v>
+        <v>187.2717899684254</v>
       </c>
       <c r="F77" t="n">
         <v>120006100</v>
@@ -2448,16 +2440,16 @@
         <v>46021</v>
       </c>
       <c r="B78" t="n">
-        <v>187.8005508490403</v>
+        <v>187.1021881103516</v>
       </c>
       <c r="C78" t="n">
-        <v>188.5487999407664</v>
+        <v>188.5488153175326</v>
       </c>
       <c r="D78" t="n">
-        <v>186.4935963146986</v>
+        <v>186.4936115238563</v>
       </c>
       <c r="E78" t="n">
-        <v>187.1021728515625</v>
+        <v>187.8005661647843</v>
       </c>
       <c r="F78" t="n">
         <v>97687300</v>
@@ -2474,7 +2466,7 @@
         <v>46022</v>
       </c>
       <c r="B79" t="n">
-        <v>189.1274459397885</v>
+        <v>186.0646057128906</v>
       </c>
       <c r="C79" t="n">
         <v>190.1151249886817</v>
@@ -2483,7 +2475,7 @@
         <v>186.0546345387688</v>
       </c>
       <c r="E79" t="n">
-        <v>186.0646057128906</v>
+        <v>189.1274459397885</v>
       </c>
       <c r="F79" t="n">
         <v>120100500</v>
@@ -2500,7 +2492,7 @@
         <v>46024</v>
       </c>
       <c r="B80" t="n">
-        <v>189.3968130035911</v>
+        <v>188.4091339111328</v>
       </c>
       <c r="C80" t="n">
         <v>192.4795957147097</v>
@@ -2509,7 +2501,7 @@
         <v>187.8204997023152</v>
       </c>
       <c r="E80" t="n">
-        <v>188.4091339111328</v>
+        <v>189.3968130035911</v>
       </c>
       <c r="F80" t="n">
         <v>148240500</v>
@@ -2526,7 +2518,7 @@
         <v>46027</v>
       </c>
       <c r="B81" t="n">
-        <v>191.3123337767646</v>
+        <v>187.6808319091797</v>
       </c>
       <c r="C81" t="n">
         <v>193.1779786425506</v>
@@ -2535,7 +2527,7 @@
         <v>185.7154296257417</v>
       </c>
       <c r="E81" t="n">
-        <v>187.6808319091797</v>
+        <v>191.3123337767646</v>
       </c>
       <c r="F81" t="n">
         <v>183529700</v>
@@ -2552,16 +2544,16 @@
         <v>46028</v>
       </c>
       <c r="B82" t="n">
-        <v>190.0752284670132</v>
+        <v>186.8029022216797</v>
       </c>
       <c r="C82" t="n">
-        <v>191.7213703933745</v>
+        <v>191.7213860539245</v>
       </c>
       <c r="D82" t="n">
-        <v>186.3838692947835</v>
+        <v>186.3838845193456</v>
       </c>
       <c r="E82" t="n">
-        <v>186.8028869628906</v>
+        <v>190.0752439930999</v>
       </c>
       <c r="F82" t="n">
         <v>176862600</v>
@@ -2578,7 +2570,7 @@
         <v>46029</v>
       </c>
       <c r="B83" t="n">
-        <v>188.1297854095839</v>
+        <v>188.6685180664062</v>
       </c>
       <c r="C83" t="n">
         <v>190.9232365533545</v>
@@ -2587,7 +2579,7 @@
         <v>186.1244680675316</v>
       </c>
       <c r="E83" t="n">
-        <v>188.6685180664062</v>
+        <v>188.1297854095839</v>
       </c>
       <c r="F83" t="n">
         <v>153543200</v>
@@ -2604,7 +2596,7 @@
         <v>46030</v>
       </c>
       <c r="B84" t="n">
-        <v>188.6685072554968</v>
+        <v>184.6080017089844</v>
       </c>
       <c r="C84" t="n">
         <v>189.1074824738404</v>
@@ -2613,7 +2605,7 @@
         <v>183.2811201033086</v>
       </c>
       <c r="E84" t="n">
-        <v>184.6080017089844</v>
+        <v>188.6685072554968</v>
       </c>
       <c r="F84" t="n">
         <v>172457000</v>
@@ -2630,7 +2622,7 @@
         <v>46031</v>
       </c>
       <c r="B85" t="n">
-        <v>184.6479238968445</v>
+        <v>184.4284362792969</v>
       </c>
       <c r="C85" t="n">
         <v>185.9049768874807</v>
@@ -2639,7 +2631,7 @@
         <v>183.2412119543349</v>
       </c>
       <c r="E85" t="n">
-        <v>184.4284362792969</v>
+        <v>184.6479238968445</v>
       </c>
       <c r="F85" t="n">
         <v>131327500</v>
@@ -2656,7 +2648,7 @@
         <v>46034</v>
       </c>
       <c r="B86" t="n">
-        <v>182.7922691735387</v>
+        <v>184.5082550048828</v>
       </c>
       <c r="C86" t="n">
         <v>186.6831584288149</v>
@@ -2665,7 +2657,7 @@
         <v>182.5927391235801</v>
       </c>
       <c r="E86" t="n">
-        <v>184.5082550048828</v>
+        <v>182.7922691735387</v>
       </c>
       <c r="F86" t="n">
         <v>137968500</v>
@@ -2682,7 +2674,7 @@
         <v>46035</v>
       </c>
       <c r="B87" t="n">
-        <v>184.5681140987238</v>
+        <v>185.376220703125</v>
       </c>
       <c r="C87" t="n">
         <v>187.6708543554723</v>
@@ -2691,7 +2683,7 @@
         <v>182.9718432388734</v>
       </c>
       <c r="E87" t="n">
-        <v>185.376220703125</v>
+        <v>184.5681140987238</v>
       </c>
       <c r="F87" t="n">
         <v>160128900</v>
@@ -2708,7 +2700,7 @@
         <v>46036</v>
       </c>
       <c r="B88" t="n">
-        <v>183.8897012556695</v>
+        <v>182.7124481201172</v>
       </c>
       <c r="C88" t="n">
         <v>184.0293738083791</v>
@@ -2717,7 +2709,7 @@
         <v>180.3779146434709</v>
       </c>
       <c r="E88" t="n">
-        <v>182.7124481201172</v>
+        <v>183.8897012556695</v>
       </c>
       <c r="F88" t="n">
         <v>159586100</v>
@@ -2734,16 +2726,16 @@
         <v>46037</v>
       </c>
       <c r="B89" t="n">
-        <v>186.0645927657271</v>
+        <v>186.6133270263672</v>
       </c>
       <c r="C89" t="n">
-        <v>189.2571189267257</v>
+        <v>189.2571344016907</v>
       </c>
       <c r="D89" t="n">
-        <v>185.8949914784577</v>
+        <v>185.895006678512</v>
       </c>
       <c r="E89" t="n">
-        <v>186.6133117675781</v>
+        <v>186.0646079796491</v>
       </c>
       <c r="F89" t="n">
         <v>206188600</v>
@@ -2760,16 +2752,16 @@
         <v>46038</v>
       </c>
       <c r="B90" t="n">
-        <v>188.6385795892923</v>
+        <v>185.7952423095703</v>
       </c>
       <c r="C90" t="n">
-        <v>189.99540517049</v>
+        <v>189.9954207742267</v>
       </c>
       <c r="D90" t="n">
-        <v>185.6455833269296</v>
+        <v>185.6455985734289</v>
       </c>
       <c r="E90" t="n">
-        <v>185.7952270507812</v>
+        <v>188.6385950815971</v>
       </c>
       <c r="F90" t="n">
         <v>187967200</v>
@@ -2786,16 +2778,16 @@
         <v>46042</v>
       </c>
       <c r="B91" t="n">
-        <v>181.4753422141945</v>
+        <v>177.6542816162109</v>
       </c>
       <c r="C91" t="n">
-        <v>181.9542325986551</v>
+        <v>181.9542169705431</v>
       </c>
       <c r="D91" t="n">
-        <v>177.1953640623503</v>
+        <v>177.1953488429791</v>
       </c>
       <c r="E91" t="n">
-        <v>177.654296875</v>
+        <v>181.4753266272146</v>
       </c>
       <c r="F91" t="n">
         <v>223345300</v>
@@ -2812,7 +2804,7 @@
         <v>46043</v>
       </c>
       <c r="B92" t="n">
-        <v>178.6320081827799</v>
+        <v>182.8920440673828</v>
       </c>
       <c r="C92" t="n">
         <v>184.9472325313386</v>
@@ -2821,7 +2813,7 @@
         <v>177.9835164834521</v>
       </c>
       <c r="E92" t="n">
-        <v>182.8920440673828</v>
+        <v>178.6320081827799</v>
       </c>
       <c r="F92" t="n">
         <v>200381000</v>
@@ -2838,7 +2830,7 @@
         <v>46044</v>
       </c>
       <c r="B93" t="n">
-        <v>184.3186915464293</v>
+        <v>184.4084777832031</v>
       </c>
       <c r="C93" t="n">
         <v>185.7353746560278</v>
@@ -2847,7 +2839,7 @@
         <v>183.5005985718231</v>
       </c>
       <c r="E93" t="n">
-        <v>184.4084777832031</v>
+        <v>184.3186915464293</v>
       </c>
       <c r="F93" t="n">
         <v>139636600</v>
@@ -2864,7 +2856,7 @@
         <v>46045</v>
       </c>
       <c r="B94" t="n">
-        <v>187.0622712594319</v>
+        <v>187.2318725585938</v>
       </c>
       <c r="C94" t="n">
         <v>189.1573747868041</v>
@@ -2873,7 +2865,7 @@
         <v>186.3838660627843</v>
       </c>
       <c r="E94" t="n">
-        <v>187.2318725585938</v>
+        <v>187.0622712594319</v>
       </c>
       <c r="F94" t="n">
         <v>142748100</v>
@@ -2890,16 +2882,16 @@
         <v>46048</v>
       </c>
       <c r="B95" t="n">
-        <v>186.7230748442759</v>
+        <v>186.03466796875</v>
       </c>
       <c r="C95" t="n">
-        <v>188.6784906596197</v>
+        <v>188.6784751839824</v>
       </c>
       <c r="D95" t="n">
-        <v>185.555808059744</v>
+        <v>185.5557928402329</v>
       </c>
       <c r="E95" t="n">
-        <v>186.0346832275391</v>
+        <v>186.7230595290241</v>
       </c>
       <c r="F95" t="n">
         <v>124799600</v>
@@ -2916,7 +2908,7 @@
         <v>46049</v>
       </c>
       <c r="B96" t="n">
-        <v>186.8028844605491</v>
+        <v>188.0798950195312</v>
       </c>
       <c r="C96" t="n">
         <v>189.5564356240106</v>
@@ -2925,7 +2917,7 @@
         <v>185.2664711415707</v>
       </c>
       <c r="E96" t="n">
-        <v>188.0798950195312</v>
+        <v>186.8028844605491</v>
       </c>
       <c r="F96" t="n">
         <v>143711600</v>
@@ -2942,7 +2934,7 @@
         <v>46050</v>
       </c>
       <c r="B97" t="n">
-        <v>190.823459633995</v>
+        <v>191.0728759765625</v>
       </c>
       <c r="C97" t="n">
         <v>191.9009400606663</v>
@@ -2951,7 +2943,7 @@
         <v>189.3967902384632</v>
       </c>
       <c r="E97" t="n">
-        <v>191.0728759765625</v>
+        <v>190.823459633995</v>
       </c>
       <c r="F97" t="n">
         <v>148552700</v>
@@ -2968,7 +2960,7 @@
         <v>46051</v>
       </c>
       <c r="B98" t="n">
-        <v>190.8933105997472</v>
+        <v>192.0605773925781</v>
       </c>
       <c r="C98" t="n">
         <v>193.0283141326731</v>
@@ -2977,7 +2969,7 @@
         <v>185.6256380470483</v>
       </c>
       <c r="E98" t="n">
-        <v>192.0605773925781</v>
+        <v>190.8933105997472</v>
       </c>
       <c r="F98" t="n">
         <v>171764400</v>
@@ -2994,7 +2986,7 @@
         <v>46052</v>
       </c>
       <c r="B99" t="n">
-        <v>190.7636224379378</v>
+        <v>190.6838073730469</v>
       </c>
       <c r="C99" t="n">
         <v>194.0359639826301</v>
@@ -3003,7 +2995,7 @@
         <v>189.0276790286862</v>
       </c>
       <c r="E99" t="n">
-        <v>190.6838073730469</v>
+        <v>190.7636224379378</v>
       </c>
       <c r="F99" t="n">
         <v>179489500</v>
@@ -3020,7 +3012,7 @@
         <v>46055</v>
       </c>
       <c r="B100" t="n">
-        <v>186.7629659025267</v>
+        <v>185.1766815185547</v>
       </c>
       <c r="C100" t="n">
         <v>189.8557348322644</v>
@@ -3029,7 +3021,7 @@
         <v>184.4483900153819</v>
       </c>
       <c r="E100" t="n">
-        <v>185.1766815185547</v>
+        <v>186.7629659025267</v>
       </c>
       <c r="F100" t="n">
         <v>165794100</v>
@@ -3046,7 +3038,7 @@
         <v>46056</v>
       </c>
       <c r="B101" t="n">
-        <v>185.8052108647954</v>
+        <v>179.9189758300781</v>
       </c>
       <c r="C101" t="n">
         <v>185.8351396091497</v>
@@ -3055,7 +3047,7 @@
         <v>175.8185703987175</v>
       </c>
       <c r="E101" t="n">
-        <v>179.9189758300781</v>
+        <v>185.8052108647954</v>
       </c>
       <c r="F101" t="n">
         <v>204019600</v>
@@ -3072,7 +3064,7 @@
         <v>46057</v>
       </c>
       <c r="B102" t="n">
-        <v>179.0410571553003</v>
+        <v>173.7833557128906</v>
       </c>
       <c r="C102" t="n">
         <v>179.1607721437711</v>
@@ -3081,7 +3073,7 @@
         <v>171.5086795929406</v>
       </c>
       <c r="E102" t="n">
-        <v>173.7833557128906</v>
+        <v>179.0410571553003</v>
       </c>
       <c r="F102" t="n">
         <v>207014100</v>
@@ -3098,7 +3090,7 @@
         <v>46058</v>
       </c>
       <c r="B103" t="n">
-        <v>174.5216119878791</v>
+        <v>171.4787445068359</v>
       </c>
       <c r="C103" t="n">
         <v>176.4072143255947</v>
@@ -3107,7 +3099,7 @@
         <v>170.6307227747363</v>
       </c>
       <c r="E103" t="n">
-        <v>171.4787445068359</v>
+        <v>174.5216119878791</v>
       </c>
       <c r="F103" t="n">
         <v>206312900</v>
@@ -3124,7 +3116,7 @@
         <v>46059</v>
       </c>
       <c r="B104" t="n">
-        <v>176.2775135166603</v>
+        <v>184.9771575927734</v>
       </c>
       <c r="C104" t="n">
         <v>186.5634420291942</v>
@@ -3133,7 +3125,7 @@
         <v>174.1923963475411</v>
       </c>
       <c r="E104" t="n">
-        <v>184.9771575927734</v>
+        <v>176.2775135166603</v>
       </c>
       <c r="F104" t="n">
         <v>231346200</v>
@@ -3150,7 +3142,7 @@
         <v>46062</v>
       </c>
       <c r="B105" t="n">
-        <v>183.8298386502086</v>
+        <v>189.5963439941406</v>
       </c>
       <c r="C105" t="n">
         <v>193.2079034382237</v>
@@ -3159,7 +3151,7 @@
         <v>183.5205647824287</v>
       </c>
       <c r="E105" t="n">
-        <v>189.5963439941406</v>
+        <v>183.8298386502086</v>
       </c>
       <c r="F105" t="n">
         <v>196387400</v>
@@ -3176,7 +3168,7 @@
         <v>46063</v>
       </c>
       <c r="B106" t="n">
-        <v>190.933219719687</v>
+        <v>188.0998382568359</v>
       </c>
       <c r="C106" t="n">
         <v>192.0306425866914</v>
@@ -3185,7 +3177,7 @@
         <v>187.6808205923615</v>
       </c>
       <c r="E106" t="n">
-        <v>188.0998382568359</v>
+        <v>190.933219719687</v>
       </c>
       <c r="F106" t="n">
         <v>136764800</v>
@@ -3202,7 +3194,7 @@
         <v>46064</v>
       </c>
       <c r="B107" t="n">
-        <v>192.0007297023972</v>
+        <v>189.6063385009766</v>
       </c>
       <c r="C107" t="n">
         <v>192.8088363522974</v>
@@ -3211,7 +3203,7 @@
         <v>188.3293278304631</v>
       </c>
       <c r="E107" t="n">
-        <v>189.6063385009766</v>
+        <v>192.0007297023972</v>
       </c>
       <c r="F107" t="n">
         <v>144192700</v>
@@ -3228,16 +3220,16 @@
         <v>46065</v>
       </c>
       <c r="B108" t="n">
-        <v>192.5793648877844</v>
+        <v>186.5036010742188</v>
       </c>
       <c r="C108" t="n">
-        <v>193.1580126884611</v>
+        <v>193.158028491682</v>
       </c>
       <c r="D108" t="n">
-        <v>186.0745817463215</v>
+        <v>186.0745969700116</v>
       </c>
       <c r="E108" t="n">
-        <v>186.5035858154297</v>
+        <v>192.5793806436633</v>
       </c>
       <c r="F108" t="n">
         <v>189932500</v>
@@ -3254,7 +3246,7 @@
         <v>46066</v>
       </c>
       <c r="B109" t="n">
-        <v>187.0423048169314</v>
+        <v>182.3832092285156</v>
       </c>
       <c r="C109" t="n">
         <v>187.0622623874058</v>
@@ -3263,7 +3255,7 @@
         <v>181.1660562233949</v>
       </c>
       <c r="E109" t="n">
-        <v>182.3832092285156</v>
+        <v>187.0423048169314</v>
       </c>
       <c r="F109" t="n">
         <v>161888000</v>
@@ -3280,16 +3272,16 @@
         <v>46070</v>
       </c>
       <c r="B110" t="n">
-        <v>181.3256935584433</v>
+        <v>184.5381927490234</v>
       </c>
       <c r="C110" t="n">
-        <v>186.7130808403767</v>
+        <v>186.7130962790006</v>
       </c>
       <c r="D110" t="n">
-        <v>178.7616860728079</v>
+        <v>178.7617008539599</v>
       </c>
       <c r="E110" t="n">
-        <v>184.5381774902344</v>
+        <v>181.3257085516038</v>
       </c>
       <c r="F110" t="n">
         <v>162276900</v>
@@ -3306,7 +3298,7 @@
         <v>46071</v>
       </c>
       <c r="B111" t="n">
-        <v>188.3093443160685</v>
+        <v>187.5411376953125</v>
       </c>
       <c r="C111" t="n">
         <v>189.9255573932224</v>
@@ -3315,7 +3307,7 @@
         <v>186.3239846890322</v>
       </c>
       <c r="E111" t="n">
-        <v>187.5411376953125</v>
+        <v>188.3093443160685</v>
       </c>
       <c r="F111" t="n">
         <v>164749100</v>
@@ -3332,16 +3324,16 @@
         <v>46072</v>
       </c>
       <c r="B112" t="n">
-        <v>186.62329889396</v>
+        <v>187.4613189697266</v>
       </c>
       <c r="C112" t="n">
-        <v>187.9900957055448</v>
+        <v>187.9900804037161</v>
       </c>
       <c r="D112" t="n">
-        <v>185.2265733363672</v>
+        <v>185.226558259481</v>
       </c>
       <c r="E112" t="n">
-        <v>187.4613342285156</v>
+        <v>186.6232837033845</v>
       </c>
       <c r="F112" t="n">
         <v>126554500</v>
@@ -3358,16 +3350,16 @@
         <v>46073</v>
       </c>
       <c r="B113" t="n">
-        <v>186.1344638821937</v>
+        <v>189.3768615722656</v>
       </c>
       <c r="C113" t="n">
-        <v>189.8856807673048</v>
+        <v>189.8856654675195</v>
       </c>
       <c r="D113" t="n">
-        <v>185.5059297314624</v>
+        <v>185.5059147845697</v>
       </c>
       <c r="E113" t="n">
-        <v>189.3768768310547</v>
+        <v>186.1344488846578</v>
       </c>
       <c r="F113" t="n">
         <v>178422300</v>
@@ -3384,7 +3376,7 @@
         <v>46076</v>
       </c>
       <c r="B114" t="n">
-        <v>190.9531547742145</v>
+        <v>191.1028137207031</v>
       </c>
       <c r="C114" t="n">
         <v>193.4972046328596</v>
@@ -3393,7 +3385,7 @@
         <v>189.1374116308485</v>
       </c>
       <c r="E114" t="n">
-        <v>191.1028137207031</v>
+        <v>190.9531547742145</v>
       </c>
       <c r="F114" t="n">
         <v>171584800</v>
@@ -3410,7 +3402,7 @@
         <v>46077</v>
       </c>
       <c r="B115" t="n">
-        <v>191.0429698590405</v>
+        <v>192.3997955322266</v>
       </c>
       <c r="C115" t="n">
         <v>193.3176459547985</v>
@@ -3419,7 +3411,7 @@
         <v>186.9625064417709</v>
       </c>
       <c r="E115" t="n">
-        <v>192.3997955322266</v>
+        <v>191.0429698590405</v>
       </c>
       <c r="F115" t="n">
         <v>175123600</v>
@@ -3436,7 +3428,7 @@
         <v>46078</v>
       </c>
       <c r="B116" t="n">
-        <v>193.9960453222018</v>
+        <v>195.1034545898438</v>
       </c>
       <c r="C116" t="n">
         <v>197.1686293956491</v>
@@ -3445,7 +3437,7 @@
         <v>193.3375824661624</v>
       </c>
       <c r="E116" t="n">
-        <v>195.1034545898438</v>
+        <v>193.9960453222018</v>
       </c>
       <c r="F116" t="n">
         <v>250637100</v>
@@ -3462,16 +3454,16 @@
         <v>46079</v>
       </c>
       <c r="B117" t="n">
-        <v>193.8164652690549</v>
+        <v>184.4583740234375</v>
       </c>
       <c r="C117" t="n">
-        <v>193.8364076167612</v>
+        <v>193.8364236513225</v>
       </c>
       <c r="D117" t="n">
-        <v>183.8896973916963</v>
+        <v>183.8897126034445</v>
       </c>
       <c r="E117" t="n">
-        <v>184.4583587646484</v>
+        <v>193.8164813019665</v>
       </c>
       <c r="F117" t="n">
         <v>360807900</v>
@@ -3488,16 +3480,16 @@
         <v>46080</v>
       </c>
       <c r="B118" t="n">
-        <v>180.8268714126474</v>
+        <v>176.7763366699219</v>
       </c>
       <c r="C118" t="n">
-        <v>182.1637395256691</v>
+        <v>182.1637238018573</v>
       </c>
       <c r="D118" t="n">
-        <v>175.9682453114839</v>
+        <v>175.9682301224481</v>
       </c>
       <c r="E118" t="n">
-        <v>176.7763519287109</v>
+        <v>180.82685580423</v>
       </c>
       <c r="F118" t="n">
         <v>311636500</v>
@@ -3514,16 +3506,16 @@
         <v>46083</v>
       </c>
       <c r="B119" t="n">
-        <v>174.601438160182</v>
+        <v>182.0539703369141</v>
       </c>
       <c r="C119" t="n">
-        <v>183.0317240302905</v>
+        <v>183.0316933488174</v>
       </c>
       <c r="D119" t="n">
-        <v>174.2323067871125</v>
+        <v>174.2322775806792</v>
       </c>
       <c r="E119" t="n">
-        <v>182.0540008544922</v>
+        <v>174.6014088918714</v>
       </c>
       <c r="F119" t="n">
         <v>209095300</v>
@@ -3540,16 +3532,16 @@
         <v>46084</v>
       </c>
       <c r="B120" t="n">
-        <v>178.0732983803544</v>
+        <v>179.6296691894531</v>
       </c>
       <c r="C120" t="n">
-        <v>180.4776603660684</v>
+        <v>180.4776756968921</v>
       </c>
       <c r="D120" t="n">
-        <v>176.5069564334623</v>
+        <v>176.5069714269912</v>
       </c>
       <c r="E120" t="n">
-        <v>179.6296539306641</v>
+        <v>178.0733135069376</v>
       </c>
       <c r="F120" t="n">
         <v>178099400</v>
@@ -3566,7 +3558,7 @@
         <v>46085</v>
       </c>
       <c r="B121" t="n">
-        <v>180.0187649948852</v>
+        <v>182.6126861572266</v>
       </c>
       <c r="C121" t="n">
         <v>184.2688145383873</v>
@@ -3575,7 +3567,7 @@
         <v>179.6396472340209</v>
       </c>
       <c r="E121" t="n">
-        <v>182.6126861572266</v>
+        <v>180.0187649948852</v>
       </c>
       <c r="F121" t="n">
         <v>177731200</v>
@@ -3592,7 +3584,7 @@
         <v>46086</v>
       </c>
       <c r="B122" t="n">
-        <v>180.7470399397241</v>
+        <v>182.9119720458984</v>
       </c>
       <c r="C122" t="n">
         <v>183.6302923567135</v>
@@ -3601,7 +3593,7 @@
         <v>177.4647274492447</v>
       </c>
       <c r="E122" t="n">
-        <v>182.9119720458984</v>
+        <v>180.7470399397241</v>
       </c>
       <c r="F122" t="n">
         <v>198779700</v>
@@ -3618,16 +3610,16 @@
         <v>46087</v>
       </c>
       <c r="B123" t="n">
-        <v>179.4201653790109</v>
+        <v>177.4048767089844</v>
       </c>
       <c r="C123" t="n">
-        <v>182.3333469017365</v>
+        <v>182.3333312190456</v>
       </c>
       <c r="D123" t="n">
-        <v>176.4072264371208</v>
+        <v>176.407211264142</v>
       </c>
       <c r="E123" t="n">
-        <v>177.4048919677734</v>
+        <v>179.420149946886</v>
       </c>
       <c r="F123" t="n">
         <v>189021900</v>
@@ -3644,7 +3636,7 @@
         <v>46090</v>
       </c>
       <c r="B124" t="n">
-        <v>176.4171820751478</v>
+        <v>182.2235870361328</v>
       </c>
       <c r="C124" t="n">
         <v>182.4829897940845</v>
@@ -3653,7 +3645,7 @@
         <v>175.1501427003192</v>
       </c>
       <c r="E124" t="n">
-        <v>182.2235870361328</v>
+        <v>176.4171820751478</v>
       </c>
       <c r="F124" t="n">
         <v>177213600</v>
@@ -3670,16 +3662,16 @@
         <v>46091</v>
       </c>
       <c r="B125" t="n">
-        <v>181.9741609804723</v>
+        <v>184.3386535644531</v>
       </c>
       <c r="C125" t="n">
-        <v>186.0047376795775</v>
+        <v>186.0047530762794</v>
       </c>
       <c r="D125" t="n">
-        <v>181.5850720874406</v>
+        <v>181.5850871183009</v>
       </c>
       <c r="E125" t="n">
-        <v>184.3386383056641</v>
+        <v>181.9741760435397</v>
       </c>
       <c r="F125" t="n">
         <v>179118500</v>
@@ -3696,7 +3688,7 @@
         <v>46092</v>
       </c>
       <c r="B126" t="n">
-        <v>185.4860219488843</v>
+        <v>185.6057434082031</v>
       </c>
       <c r="C126" t="n">
         <v>187.1921136401388</v>
@@ -3705,7 +3697,7 @@
         <v>184.0293448898806</v>
       </c>
       <c r="E126" t="n">
-        <v>185.6057434082031</v>
+        <v>185.4860219488843</v>
       </c>
       <c r="F126" t="n">
         <v>145280400</v>
@@ -3722,16 +3714,16 @@
         <v>46093</v>
       </c>
       <c r="B127" t="n">
-        <v>183.6302794851663</v>
+        <v>182.7223358154297</v>
       </c>
       <c r="C127" t="n">
-        <v>184.5182492431283</v>
+        <v>184.5182338343672</v>
       </c>
       <c r="D127" t="n">
-        <v>181.3355215595592</v>
+        <v>181.3355064165816</v>
       </c>
       <c r="E127" t="n">
-        <v>182.7223510742188</v>
+        <v>183.6302641505579</v>
       </c>
       <c r="F127" t="n">
         <v>155762700</v>
@@ -3748,16 +3740,16 @@
         <v>46094</v>
       </c>
       <c r="B128" t="n">
-        <v>184.4982761588831</v>
+        <v>179.8389434814453</v>
       </c>
       <c r="C128" t="n">
-        <v>185.6656060713691</v>
+        <v>185.6656218245341</v>
       </c>
       <c r="D128" t="n">
-        <v>179.5296376335348</v>
+        <v>179.5296528660815</v>
       </c>
       <c r="E128" t="n">
-        <v>179.8389282226562</v>
+        <v>184.4982918130038</v>
       </c>
       <c r="F128" t="n">
         <v>160988400</v>
@@ -3774,16 +3766,16 @@
         <v>46097</v>
       </c>
       <c r="B129" t="n">
-        <v>182.5527399223597</v>
+        <v>182.8021545410156</v>
       </c>
       <c r="C129" t="n">
-        <v>188.4492658789173</v>
+        <v>188.4492501487561</v>
       </c>
       <c r="D129" t="n">
-        <v>180.9962999229416</v>
+        <v>180.9962848148914</v>
       </c>
       <c r="E129" t="n">
-        <v>182.8021697998047</v>
+        <v>182.5527246843909</v>
       </c>
       <c r="F129" t="n">
         <v>217307400</v>
@@ -3800,16 +3792,16 @@
         <v>46098</v>
       </c>
       <c r="B130" t="n">
-        <v>184.6379576703901</v>
+        <v>181.5151062011719</v>
       </c>
       <c r="C130" t="n">
-        <v>184.9771786272242</v>
+        <v>184.9771941770484</v>
       </c>
       <c r="D130" t="n">
-        <v>181.2656610816535</v>
+        <v>181.2656763194747</v>
       </c>
       <c r="E130" t="n">
-        <v>181.5150909423828</v>
+        <v>184.6379731916982</v>
       </c>
       <c r="F130" t="n">
         <v>182497800</v>
@@ -3826,7 +3818,7 @@
         <v>46099</v>
       </c>
       <c r="B131" t="n">
-        <v>182.0638447517288</v>
+        <v>179.9885864257812</v>
       </c>
       <c r="C131" t="n">
         <v>182.9618014097589</v>
@@ -3835,7 +3827,7 @@
         <v>179.9187539793071</v>
       </c>
       <c r="E131" t="n">
-        <v>179.9885864257812</v>
+        <v>182.0638447517288</v>
       </c>
       <c r="F131" t="n">
         <v>156683100</v>
@@ -3852,16 +3844,16 @@
         <v>46100</v>
       </c>
       <c r="B132" t="n">
-        <v>177.6040375011918</v>
+        <v>178.1527709960938</v>
       </c>
       <c r="C132" t="n">
-        <v>179.569546076418</v>
+        <v>179.5695306962835</v>
       </c>
       <c r="D132" t="n">
-        <v>175.3890990582871</v>
+        <v>175.3890840362079</v>
       </c>
       <c r="E132" t="n">
-        <v>178.1527862548828</v>
+        <v>177.6040222894031</v>
       </c>
       <c r="F132" t="n">
         <v>170968500</v>
@@ -3878,16 +3870,16 @@
         <v>46101</v>
       </c>
       <c r="B133" t="n">
-        <v>177.5940529420793</v>
+        <v>172.30615234375</v>
       </c>
       <c r="C133" t="n">
-        <v>177.8534545050662</v>
+        <v>177.853470255105</v>
       </c>
       <c r="D133" t="n">
-        <v>171.3283763370981</v>
+        <v>171.3283915093003</v>
       </c>
       <c r="E133" t="n">
-        <v>172.3061370849609</v>
+        <v>177.5940686691464</v>
       </c>
       <c r="F133" t="n">
         <v>241323500</v>
@@ -3904,7 +3896,7 @@
         <v>46104</v>
       </c>
       <c r="B134" t="n">
-        <v>176.8557415306554</v>
+        <v>175.2394409179688</v>
       </c>
       <c r="C134" t="n">
         <v>177.9632107122345</v>
@@ -3913,7 +3905,7 @@
         <v>174.3614429436745</v>
       </c>
       <c r="E134" t="n">
-        <v>175.2394409179688</v>
+        <v>176.8557415306554</v>
       </c>
       <c r="F134" t="n">
         <v>182836300</v>
@@ -3930,7 +3922,7 @@
         <v>46105</v>
       </c>
       <c r="B135" t="n">
-        <v>174.4312942297872</v>
+        <v>174.8004455566406</v>
       </c>
       <c r="C135" t="n">
         <v>175.8181236639554</v>
@@ -3939,7 +3931,7 @@
         <v>173.5832266030264</v>
       </c>
       <c r="E135" t="n">
-        <v>174.8004455566406</v>
+        <v>174.4312942297872</v>
       </c>
       <c r="F135" t="n">
         <v>147667800</v>
@@ -3956,7 +3948,7 @@
         <v>46106</v>
       </c>
       <c r="B136" t="n">
-        <v>176.6961233561449</v>
+        <v>178.2725067138672</v>
       </c>
       <c r="C136" t="n">
         <v>180.8067226806179</v>
@@ -3965,7 +3957,7 @@
         <v>176.4466934898736</v>
       </c>
       <c r="E136" t="n">
-        <v>178.2725067138672</v>
+        <v>176.6961233561449</v>
       </c>
       <c r="F136" t="n">
         <v>162602100</v>
@@ -3982,7 +3974,7 @@
         <v>46107</v>
       </c>
       <c r="B137" t="n">
-        <v>175.6684741654964</v>
+        <v>170.8494873046875</v>
       </c>
       <c r="C137" t="n">
         <v>176.1074579435819</v>
@@ -3991,7 +3983,7 @@
         <v>170.7497092682189</v>
       </c>
       <c r="E137" t="n">
-        <v>170.8494873046875</v>
+        <v>175.6684741654964</v>
       </c>
       <c r="F137" t="n">
         <v>186152200</v>
@@ -4008,16 +4000,16 @@
         <v>46108</v>
       </c>
       <c r="B138" t="n">
-        <v>169.6122945102883</v>
+        <v>167.1379699707031</v>
       </c>
       <c r="C138" t="n">
-        <v>170.5800835262955</v>
+        <v>170.5800990993323</v>
       </c>
       <c r="D138" t="n">
-        <v>166.6291080850299</v>
+        <v>166.629123297364</v>
       </c>
       <c r="E138" t="n">
-        <v>167.1379547119141</v>
+        <v>169.6123099949711</v>
       </c>
       <c r="F138" t="n">
         <v>196212700</v>
@@ -4034,7 +4026,7 @@
         <v>46111</v>
       </c>
       <c r="B139" t="n">
-        <v>168.3950875250076</v>
+        <v>164.7933197021484</v>
       </c>
       <c r="C139" t="n">
         <v>169.0635577295173</v>
@@ -4043,7 +4035,7 @@
         <v>163.8953782868944</v>
       </c>
       <c r="E139" t="n">
-        <v>164.7933197021484</v>
+        <v>168.3950875250076</v>
       </c>
       <c r="F139" t="n">
         <v>185627000</v>
@@ -4060,16 +4052,16 @@
         <v>46112</v>
       </c>
       <c r="B140" t="n">
-        <v>166.5892250311153</v>
+        <v>174.0022583007812</v>
       </c>
       <c r="C140" t="n">
-        <v>174.2217730660379</v>
+        <v>174.2217577880002</v>
       </c>
       <c r="D140" t="n">
-        <v>166.5792533168182</v>
+        <v>166.5792387089764</v>
       </c>
       <c r="E140" t="n">
-        <v>174.0022735595703</v>
+        <v>166.589210422399</v>
       </c>
       <c r="F140" t="n">
         <v>226181300</v>
@@ -4086,16 +4078,16 @@
         <v>46113</v>
       </c>
       <c r="B141" t="n">
-        <v>175.5986272559566</v>
+        <v>175.3491821289062</v>
       </c>
       <c r="C141" t="n">
-        <v>176.9654980623514</v>
+        <v>176.9654826629128</v>
       </c>
       <c r="D141" t="n">
-        <v>174.3514779146501</v>
+        <v>174.351462742682</v>
       </c>
       <c r="E141" t="n">
-        <v>175.3491973876953</v>
+        <v>175.5986119754623</v>
       </c>
       <c r="F141" t="n">
         <v>168132000</v>
@@ -4112,16 +4104,16 @@
         <v>46114</v>
       </c>
       <c r="B142" t="n">
-        <v>171.7873183615289</v>
+        <v>176.9854583740234</v>
       </c>
       <c r="C142" t="n">
-        <v>177.0852211444685</v>
+        <v>177.0852364118599</v>
       </c>
       <c r="D142" t="n">
-        <v>170.9791680862979</v>
+        <v>170.9791828272563</v>
       </c>
       <c r="E142" t="n">
-        <v>176.9854431152344</v>
+        <v>171.787333172162</v>
       </c>
       <c r="F142" t="n">
         <v>143143200</v>
@@ -4138,7 +4130,7 @@
         <v>46118</v>
       </c>
       <c r="B143" t="n">
-        <v>176.7559774774269</v>
+        <v>177.2348785400391</v>
       </c>
       <c r="C143" t="n">
         <v>177.3845303646084</v>
@@ -4147,7 +4139,7 @@
         <v>175.3591611441553</v>
       </c>
       <c r="E143" t="n">
-        <v>177.2348785400391</v>
+        <v>176.7559774774269</v>
       </c>
       <c r="F143" t="n">
         <v>107564300</v>
@@ -4164,7 +4156,7 @@
         <v>46119</v>
       </c>
       <c r="B144" t="n">
-        <v>175.3292270516068</v>
+        <v>177.6938323974609</v>
       </c>
       <c r="C144" t="n">
         <v>177.8235255680002</v>
@@ -4173,7 +4165,7 @@
         <v>173.2639557965079</v>
       </c>
       <c r="E144" t="n">
-        <v>177.6938323974609</v>
+        <v>175.3292270516068</v>
       </c>
       <c r="F144" t="n">
         <v>132534900</v>
@@ -4190,7 +4182,7 @@
         <v>46120</v>
       </c>
       <c r="B145" t="n">
-        <v>184.079243714486</v>
+        <v>181.6647644042969</v>
       </c>
       <c r="C145" t="n">
         <v>184.837505037226</v>
@@ -4199,7 +4191,7 @@
         <v>179.8888249511496</v>
       </c>
       <c r="E145" t="n">
-        <v>181.6647644042969</v>
+        <v>184.079243714486</v>
       </c>
       <c r="F145" t="n">
         <v>147732700</v>
@@ -4216,16 +4208,16 @@
         <v>46121</v>
       </c>
       <c r="B146" t="n">
-        <v>181.4252987848774</v>
+        <v>183.4906005859375</v>
       </c>
       <c r="C146" t="n">
-        <v>183.6601958045732</v>
+        <v>183.6602110774668</v>
       </c>
       <c r="D146" t="n">
-        <v>180.2080798537204</v>
+        <v>180.2080948395415</v>
       </c>
       <c r="E146" t="n">
-        <v>183.4905853271484</v>
+        <v>181.4253138719204</v>
       </c>
       <c r="F146" t="n">
         <v>116428500</v>
@@ -4242,7 +4234,7 @@
         <v>46122</v>
       </c>
       <c r="B147" t="n">
-        <v>183.8896736698189</v>
+        <v>188.1998291015625</v>
       </c>
       <c r="C147" t="n">
         <v>189.5666999081706</v>
@@ -4251,7 +4243,7 @@
         <v>183.8797019557237</v>
       </c>
       <c r="E147" t="n">
-        <v>188.1998291015625</v>
+        <v>183.8896736698189</v>
       </c>
       <c r="F147" t="n">
         <v>160459500</v>
@@ -4268,7 +4260,7 @@
         <v>46125</v>
       </c>
       <c r="B148" t="n">
-        <v>185.605746824658</v>
+        <v>188.8782653808594</v>
       </c>
       <c r="C148" t="n">
         <v>189.2274732756209</v>
@@ -4277,7 +4269,7 @@
         <v>185.3164148846483</v>
       </c>
       <c r="E148" t="n">
-        <v>188.8782653808594</v>
+        <v>185.605746824658</v>
       </c>
       <c r="F148" t="n">
         <v>133648200</v>
@@ -4294,7 +4286,7 @@
         <v>46126</v>
       </c>
       <c r="B149" t="n">
-        <v>190.4047764107204</v>
+        <v>196.0618438720703</v>
       </c>
       <c r="C149" t="n">
         <v>196.0618438720703</v>
@@ -4303,7 +4295,7 @@
         <v>190.3349439656124</v>
       </c>
       <c r="E149" t="n">
-        <v>196.0618438720703</v>
+        <v>190.4047764107204</v>
       </c>
       <c r="F149" t="n">
         <v>161307000</v>
@@ -4320,7 +4312,7 @@
         <v>46127</v>
       </c>
       <c r="B150" t="n">
-        <v>196.0917851116163</v>
+        <v>198.4164733886719</v>
       </c>
       <c r="C150" t="n">
         <v>199.9429830157183</v>
@@ -4329,7 +4321,7 @@
         <v>195.2936216855987</v>
       </c>
       <c r="E150" t="n">
-        <v>198.4164733886719</v>
+        <v>196.0917851116163</v>
       </c>
       <c r="F150" t="n">
         <v>185338400</v>
@@ -4346,7 +4338,7 @@
         <v>46128</v>
       </c>
       <c r="B151" t="n">
-        <v>196.9797440092329</v>
+        <v>197.8976593017578</v>
       </c>
       <c r="C151" t="n">
         <v>199.3942384790618</v>
@@ -4355,7 +4347,7 @@
         <v>195.3634433694217</v>
       </c>
       <c r="E151" t="n">
-        <v>197.8976593017578</v>
+        <v>196.9797440092329</v>
       </c>
       <c r="F151" t="n">
         <v>134012900</v>
@@ -4372,7 +4364,7 @@
         <v>46129</v>
       </c>
       <c r="B152" t="n">
-        <v>199.444107632571</v>
+        <v>201.2200469970703</v>
       </c>
       <c r="C152" t="n">
         <v>201.2400056483541</v>
@@ -4381,7 +4373,7 @@
         <v>198.8155547450397</v>
       </c>
       <c r="E152" t="n">
-        <v>201.2200469970703</v>
+        <v>199.444107632571</v>
       </c>
       <c r="F152" t="n">
         <v>160324400</v>
@@ -4398,7 +4390,7 @@
         <v>46132</v>
       </c>
       <c r="B153" t="n">
-        <v>199.5239239232554</v>
+        <v>201.5991821289062</v>
       </c>
       <c r="C153" t="n">
         <v>201.7089318732817</v>
@@ -4407,7 +4399,7 @@
         <v>197.3888049886708</v>
       </c>
       <c r="E153" t="n">
-        <v>201.5991821289062</v>
+        <v>199.5239239232554</v>
       </c>
       <c r="F153" t="n">
         <v>119381400</v>
@@ -4424,7 +4416,7 @@
         <v>46133</v>
       </c>
       <c r="B154" t="n">
-        <v>201.6690479582887</v>
+        <v>199.4241790771484</v>
       </c>
       <c r="C154" t="n">
         <v>202.2876291783034</v>
@@ -4433,7 +4425,7 @@
         <v>198.5461810430697</v>
       </c>
       <c r="E154" t="n">
-        <v>199.4241790771484</v>
+        <v>201.6690479582887</v>
       </c>
       <c r="F154" t="n">
         <v>107945300</v>
@@ -4450,7 +4442,7 @@
         <v>46134</v>
       </c>
       <c r="B155" t="n">
-        <v>200.5316418294082</v>
+        <v>202.0381927490234</v>
       </c>
       <c r="C155" t="n">
         <v>202.0381927490234</v>
@@ -4459,7 +4451,7 @@
         <v>198.546174602744</v>
       </c>
       <c r="E155" t="n">
-        <v>202.0381927490234</v>
+        <v>200.5316418294082</v>
       </c>
       <c r="F155" t="n">
         <v>107501000</v>
@@ -4476,7 +4468,7 @@
         <v>46135</v>
       </c>
       <c r="B156" t="n">
-        <v>201.9982837593082</v>
+        <v>199.1847076416016</v>
       </c>
       <c r="C156" t="n">
         <v>203.3651545152774</v>
@@ -4485,7 +4477,7 @@
         <v>196.7702284327844</v>
       </c>
       <c r="E156" t="n">
-        <v>199.1847076416016</v>
+        <v>201.9982837593082</v>
       </c>
       <c r="F156" t="n">
         <v>113561800</v>
@@ -4502,7 +4494,7 @@
         <v>46136</v>
       </c>
       <c r="B157" t="n">
-        <v>199.5039827094276</v>
+        <v>207.7950286865234</v>
       </c>
       <c r="C157" t="n">
         <v>210.468909435165</v>
@@ -4511,7 +4503,7 @@
         <v>199.3543156614425</v>
       </c>
       <c r="E157" t="n">
-        <v>207.7950286865234</v>
+        <v>199.5039827094276</v>
       </c>
       <c r="F157" t="n">
         <v>214134400</v>
@@ -4528,7 +4520,7 @@
         <v>46139</v>
       </c>
       <c r="B158" t="n">
-        <v>209.1718784416434</v>
+        <v>216.1160125732422</v>
       </c>
       <c r="C158" t="n">
         <v>216.335512072091</v>
@@ -4537,7 +4529,7 @@
         <v>206.9070662315077</v>
       </c>
       <c r="E158" t="n">
-        <v>216.1160125732422</v>
+        <v>209.1718784416434</v>
       </c>
       <c r="F158" t="n">
         <v>187172400</v>
@@ -4554,7 +4546,7 @@
         <v>46140</v>
       </c>
       <c r="B159" t="n">
-        <v>209.0122528840405</v>
+        <v>212.6838531494141</v>
       </c>
       <c r="C159" t="n">
         <v>214.2402930542568</v>
@@ -4563,7 +4555,7 @@
         <v>207.7251862691963</v>
       </c>
       <c r="E159" t="n">
-        <v>212.6838531494141</v>
+        <v>209.0122528840405</v>
       </c>
       <c r="F159" t="n">
         <v>180275400</v>
@@ -4580,7 +4572,7 @@
         <v>46141</v>
       </c>
       <c r="B160" t="n">
-        <v>212.2149257168926</v>
+        <v>208.7727966308594</v>
       </c>
       <c r="C160" t="n">
         <v>212.2348843687743</v>
@@ -4589,7 +4581,7 @@
         <v>207.1066069625242</v>
       </c>
       <c r="E160" t="n">
-        <v>208.7727966308594</v>
+        <v>212.2149257168926</v>
       </c>
       <c r="F160" t="n">
         <v>123711800</v>
@@ -4606,16 +4598,16 @@
         <v>46142</v>
       </c>
       <c r="B161" t="n">
-        <v>209.4512425942353</v>
+        <v>199.1148681640625</v>
       </c>
       <c r="C161" t="n">
-        <v>209.820409153207</v>
+        <v>209.8203930740204</v>
       </c>
       <c r="D161" t="n">
-        <v>198.2468571251534</v>
+        <v>198.2468419328838</v>
       </c>
       <c r="E161" t="n">
-        <v>199.1148834228516</v>
+        <v>209.4512265433391</v>
       </c>
       <c r="F161" t="n">
         <v>225239200</v>
@@ -4632,16 +4624,16 @@
         <v>46143</v>
       </c>
       <c r="B162" t="n">
-        <v>200.8209691272831</v>
+        <v>197.9974365234375</v>
       </c>
       <c r="C162" t="n">
-        <v>202.5370477944956</v>
+        <v>202.5370634031337</v>
       </c>
       <c r="D162" t="n">
-        <v>196.6704525729091</v>
+        <v>196.6704677294345</v>
       </c>
       <c r="E162" t="n">
-        <v>197.9974212646484</v>
+        <v>200.8209846036705</v>
       </c>
       <c r="F162" t="n">
         <v>128647000</v>
@@ -4658,7 +4650,7 @@
         <v>46146</v>
       </c>
       <c r="B163" t="n">
-        <v>199.0450218084295</v>
+        <v>198.02734375</v>
       </c>
       <c r="C163" t="n">
         <v>201.2699318245734</v>
@@ -4667,7 +4659,7 @@
         <v>194.2958829090753</v>
       </c>
       <c r="E163" t="n">
-        <v>198.02734375</v>
+        <v>199.0450218084295</v>
       </c>
       <c r="F163" t="n">
         <v>125368100</v>
@@ -4684,7 +4676,7 @@
         <v>46147</v>
       </c>
       <c r="B164" t="n">
-        <v>198.8454820247872</v>
+        <v>196.0518646240234</v>
       </c>
       <c r="C164" t="n">
         <v>199.7833407086998</v>
@@ -4693,7 +4685,7 @@
         <v>195.5829352820671</v>
       </c>
       <c r="E164" t="n">
-        <v>196.0518646240234</v>
+        <v>198.8454820247872</v>
       </c>
       <c r="F164" t="n">
         <v>113406600</v>
@@ -4710,7 +4702,7 @@
         <v>46148</v>
       </c>
       <c r="B165" t="n">
-        <v>199.4341385249406</v>
+        <v>207.3560333251953</v>
       </c>
       <c r="C165" t="n">
         <v>207.7950323152332</v>
@@ -4719,7 +4711,7 @@
         <v>198.1570588579161</v>
       </c>
       <c r="E165" t="n">
-        <v>207.3560333251953</v>
+        <v>199.4341385249406</v>
       </c>
       <c r="F165" t="n">
         <v>188362800</v>
@@ -4736,7 +4728,7 @@
         <v>46149</v>
       </c>
       <c r="B166" t="n">
-        <v>207.8648724722903</v>
+        <v>211.0176696777344</v>
       </c>
       <c r="C166" t="n">
         <v>213.7115092245668</v>
@@ -4745,7 +4737,7 @@
         <v>206.0290722858257</v>
       </c>
       <c r="E166" t="n">
-        <v>211.0176696777344</v>
+        <v>207.8648724722903</v>
       </c>
       <c r="F166" t="n">
         <v>168307900</v>
@@ -4762,7 +4754,7 @@
         <v>46150</v>
       </c>
       <c r="B167" t="n">
-        <v>212.5441790763045</v>
+        <v>214.709228515625</v>
       </c>
       <c r="C167" t="n">
         <v>217.3033052467507</v>
@@ -4771,7 +4763,7 @@
         <v>212.4044989584125</v>
       </c>
       <c r="E167" t="n">
-        <v>214.709228515625</v>
+        <v>212.5441790763045</v>
       </c>
       <c r="F167" t="n">
         <v>136421400</v>
@@ -4788,7 +4780,7 @@
         <v>46153</v>
       </c>
       <c r="B168" t="n">
-        <v>213.5518657378577</v>
+        <v>218.9395599365234</v>
       </c>
       <c r="C168" t="n">
         <v>221.7930381906342</v>
@@ -4797,7 +4789,7 @@
         <v>213.402213909002</v>
       </c>
       <c r="E168" t="n">
-        <v>218.9395599365234</v>
+        <v>213.5518657378577</v>
       </c>
       <c r="F168" t="n">
         <v>160685800</v>
@@ -4814,7 +4806,7 @@
         <v>46154</v>
       </c>
       <c r="B169" t="n">
-        <v>218.0515943496244</v>
+        <v>220.2765045166016</v>
       </c>
       <c r="C169" t="n">
         <v>223.239732575863</v>
@@ -4823,7 +4815,7 @@
         <v>214.4298677829735</v>
       </c>
       <c r="E169" t="n">
-        <v>220.2765045166016</v>
+        <v>218.0515943496244</v>
       </c>
       <c r="F169" t="n">
         <v>159176600</v>
@@ -4840,7 +4832,7 @@
         <v>46155</v>
       </c>
       <c r="B170" t="n">
-        <v>224.4170305354026</v>
+        <v>225.3149871826172</v>
       </c>
       <c r="C170" t="n">
         <v>227.3203978139454</v>
@@ -4849,7 +4841,7 @@
         <v>221.0647077692387</v>
       </c>
       <c r="E170" t="n">
-        <v>225.3149871826172</v>
+        <v>224.4170305354026</v>
       </c>
       <c r="F170" t="n">
         <v>150405400</v>
@@ -4866,7 +4858,7 @@
         <v>46156</v>
       </c>
       <c r="B171" t="n">
-        <v>229.3258255277811</v>
+        <v>235.202392578125</v>
       </c>
       <c r="C171" t="n">
         <v>236.0005559723521</v>
@@ -4875,7 +4867,7 @@
         <v>228.7770767762568</v>
       </c>
       <c r="E171" t="n">
-        <v>235.202392578125</v>
+        <v>229.3258255277811</v>
       </c>
       <c r="F171" t="n">
         <v>180782900</v>
@@ -4892,16 +4884,16 @@
         <v>46157</v>
       </c>
       <c r="B172" t="n">
-        <v>229.2360294447337</v>
+        <v>224.80615234375</v>
       </c>
       <c r="C172" t="n">
-        <v>230.9720668751014</v>
+        <v>230.9720511978</v>
       </c>
       <c r="D172" t="n">
-        <v>223.7286287034134</v>
+        <v>223.7286135177626</v>
       </c>
       <c r="E172" t="n">
-        <v>224.8061676025391</v>
+        <v>229.2360138852663</v>
       </c>
       <c r="F172" t="n">
         <v>180977600</v>
@@ -4918,7 +4910,7 @@
         <v>46160</v>
       </c>
       <c r="B173" t="n">
-        <v>229.345773483712</v>
+        <v>221.8130035400391</v>
       </c>
       <c r="C173" t="n">
         <v>229.4754818886306</v>
@@ -4927,7 +4919,7 @@
         <v>217.8719993892805</v>
       </c>
       <c r="E173" t="n">
-        <v>221.8130035400391</v>
+        <v>229.345773483712</v>
       </c>
       <c r="F173" t="n">
         <v>146280900</v>
@@ -4944,7 +4936,7 @@
         <v>46161</v>
       </c>
       <c r="B174" t="n">
-        <v>219.1191400841904</v>
+        <v>220.1068878173828</v>
       </c>
       <c r="C174" t="n">
         <v>223.9680572056967</v>
@@ -4953,7 +4945,7 @@
         <v>217.4130483552105</v>
       </c>
       <c r="E174" t="n">
-        <v>220.1068878173828</v>
+        <v>219.1191400841904</v>
       </c>
       <c r="F174" t="n">
         <v>140948200</v>
@@ -4970,7 +4962,7 @@
         <v>46162</v>
       </c>
       <c r="B175" t="n">
-        <v>222.6710257508039</v>
+        <v>222.9603729248047</v>
       </c>
       <c r="C175" t="n">
         <v>225.6143103895453</v>
@@ -4979,7 +4971,7 @@
         <v>219.9971448577806</v>
       </c>
       <c r="E175" t="n">
-        <v>222.9603729248047</v>
+        <v>222.6710257508039</v>
       </c>
       <c r="F175" t="n">
         <v>184201600</v>
@@ -4996,7 +4988,7 @@
         <v>46163</v>
       </c>
       <c r="B176" t="n">
-        <v>221.7830583738447</v>
+        <v>219.0093994140625</v>
       </c>
       <c r="C176" t="n">
         <v>226.8814055684356</v>
@@ -5005,7 +4997,7 @@
         <v>217.4330007955402</v>
       </c>
       <c r="E176" t="n">
-        <v>219.0093994140625</v>
+        <v>221.7830583738447</v>
       </c>
       <c r="F176" t="n">
         <v>203381800</v>
@@ -5022,7 +5014,7 @@
         <v>46164</v>
       </c>
       <c r="B177" t="n">
-        <v>220.3962175709585</v>
+        <v>214.8389282226562</v>
       </c>
       <c r="C177" t="n">
         <v>220.5059673180016</v>
@@ -5031,7 +5023,7 @@
         <v>214.3101381389001</v>
       </c>
       <c r="E177" t="n">
-        <v>214.8389282226562</v>
+        <v>220.3962175709585</v>
       </c>
       <c r="F177" t="n">
         <v>169275700</v>
@@ -5048,7 +5040,7 @@
         <v>46168</v>
       </c>
       <c r="B178" t="n">
-        <v>216.0461718127993</v>
+        <v>214.3700103759766</v>
       </c>
       <c r="C178" t="n">
         <v>217.6824311685512</v>
@@ -5057,7 +5049,7 @@
         <v>211.5165320236786</v>
       </c>
       <c r="E178" t="n">
-        <v>214.3700103759766</v>
+        <v>216.0461718127993</v>
       </c>
       <c r="F178" t="n">
         <v>187202600</v>
@@ -5074,7 +5066,7 @@
         <v>46169</v>
       </c>
       <c r="B179" t="n">
-        <v>213.6316806617713</v>
+        <v>212.1151580810547</v>
       </c>
       <c r="C179" t="n">
         <v>213.6616110269177</v>
@@ -5083,7 +5075,7 @@
         <v>208.3038625298546</v>
       </c>
       <c r="E179" t="n">
-        <v>212.1151580810547</v>
+        <v>213.6316806617713</v>
       </c>
       <c r="F179" t="n">
         <v>167601200</v>
@@ -5100,16 +5092,16 @@
         <v>46170</v>
       </c>
       <c r="B180" t="n">
-        <v>210.7981551984497</v>
+        <v>213.7613983154297</v>
       </c>
       <c r="C180" t="n">
-        <v>215.0284909668814</v>
+        <v>215.0285063161196</v>
       </c>
       <c r="D180" t="n">
-        <v>210.7382944698381</v>
+        <v>210.738309512832</v>
       </c>
       <c r="E180" t="n">
-        <v>213.7613830566406</v>
+        <v>210.7981702457166</v>
       </c>
       <c r="F180" t="n">
         <v>143996000</v>
@@ -5126,7 +5118,7 @@
         <v>46171</v>
       </c>
       <c r="B181" t="n">
-        <v>214.0906505321041</v>
+        <v>210.6584930419922</v>
       </c>
       <c r="C181" t="n">
         <v>217.3631692496548</v>
@@ -5135,7 +5127,7 @@
         <v>210.6485213277038</v>
       </c>
       <c r="E181" t="n">
-        <v>210.6584930419922</v>
+        <v>214.0906505321041</v>
       </c>
       <c r="F181" t="n">
         <v>289410600</v>
@@ -5152,7 +5144,7 @@
         <v>46174</v>
       </c>
       <c r="B182" t="n">
-        <v>215.2380189209027</v>
+        <v>223.8483428955078</v>
       </c>
       <c r="C182" t="n">
         <v>224.3571743491113</v>
@@ -5161,7 +5153,7 @@
         <v>215.2080885544549</v>
       </c>
       <c r="E182" t="n">
-        <v>223.8483428955078</v>
+        <v>215.2380189209027</v>
       </c>
       <c r="F182" t="n">
         <v>212850700</v>
@@ -5178,7 +5170,7 @@
         <v>46175</v>
       </c>
       <c r="B183" t="n">
-        <v>226.6618858382332</v>
+        <v>222.3118438720703</v>
       </c>
       <c r="C183" t="n">
         <v>231.7502608645459</v>
@@ -5187,7 +5179,7 @@
         <v>220.8451951370975</v>
       </c>
       <c r="E183" t="n">
-        <v>222.3118438720703</v>
+        <v>226.6618858382332</v>
       </c>
       <c r="F183" t="n">
         <v>193362900</v>
@@ -5204,7 +5196,7 @@
         <v>46176</v>
       </c>
       <c r="B184" t="n">
-        <v>221.2143597561905</v>
+        <v>214.26025390625</v>
       </c>
       <c r="C184" t="n">
         <v>222.3118572511273</v>
@@ -5213,7 +5205,7 @@
         <v>214.0207957553572</v>
       </c>
       <c r="E184" t="n">
-        <v>214.26025390625</v>
+        <v>221.2143597561905</v>
       </c>
       <c r="F184" t="n">
         <v>160907000</v>
@@ -5230,7 +5222,7 @@
         <v>46177</v>
       </c>
       <c r="B185" t="n">
-        <v>213.6709127939037</v>
+        <v>218.4156036376953</v>
       </c>
       <c r="C185" t="n">
         <v>221.3523199881091</v>
@@ -5239,7 +5231,7 @@
         <v>210.73419644349</v>
       </c>
       <c r="E185" t="n">
-        <v>218.4156036376953</v>
+        <v>213.6709127939037</v>
       </c>
       <c r="F185" t="n">
         <v>169022200</v>
@@ -5256,7 +5248,7 @@
         <v>46178</v>
       </c>
       <c r="B186" t="n">
-        <v>214.2902104723603</v>
+        <v>204.8707580566406</v>
       </c>
       <c r="C186" t="n">
         <v>214.6298267834636</v>
@@ -5265,7 +5257,7 @@
         <v>204.101614447126</v>
       </c>
       <c r="E186" t="n">
-        <v>204.8707580566406</v>
+        <v>214.2902104723603</v>
       </c>
       <c r="F186" t="n">
         <v>219655500</v>
@@ -5282,7 +5274,7 @@
         <v>46181</v>
       </c>
       <c r="B187" t="n">
-        <v>209.9450713288228</v>
+        <v>208.4067993164062</v>
       </c>
       <c r="C187" t="n">
         <v>210.2347557268212</v>
@@ -5291,7 +5283,7 @@
         <v>205.7697506938822</v>
       </c>
       <c r="E187" t="n">
-        <v>208.4067993164062</v>
+        <v>209.9450713288228</v>
       </c>
       <c r="F187" t="n">
         <v>138372800</v>
@@ -5308,7 +5300,7 @@
         <v>46182</v>
       </c>
       <c r="B188" t="n">
-        <v>210.3845825512031</v>
+        <v>207.9573059082031</v>
       </c>
       <c r="C188" t="n">
         <v>211.1637095162451</v>
@@ -5317,7 +5309,7 @@
         <v>199.1171915656509</v>
       </c>
       <c r="E188" t="n">
-        <v>207.9573059082031</v>
+        <v>210.3845825512031</v>
       </c>
       <c r="F188" t="n">
         <v>180962500</v>
@@ -5334,7 +5326,7 @@
         <v>46183</v>
       </c>
       <c r="B189" t="n">
-        <v>204.2014963256503</v>
+        <v>200.1959838867188</v>
       </c>
       <c r="C189" t="n">
         <v>206.9883864105018</v>
@@ -5343,7 +5335,7 @@
         <v>199.696542748819</v>
       </c>
       <c r="E189" t="n">
-        <v>200.1959838867188</v>
+        <v>204.2014963256503</v>
       </c>
       <c r="F189" t="n">
         <v>161746600</v>
@@ -5360,7 +5352,7 @@
         <v>46184</v>
       </c>
       <c r="B190" t="n">
-        <v>201.2647947500858</v>
+        <v>204.6410064697266</v>
       </c>
       <c r="C190" t="n">
         <v>205.4301320010667</v>
@@ -5369,7 +5361,7 @@
         <v>199.3169621236104</v>
       </c>
       <c r="E190" t="n">
-        <v>204.6410064697266</v>
+        <v>201.2647947500858</v>
       </c>
       <c r="F190" t="n">
         <v>158643200</v>
@@ -5386,7 +5378,7 @@
         <v>46185</v>
       </c>
       <c r="B191" t="n">
-        <v>204.6310298517525</v>
+        <v>204.9606628417969</v>
       </c>
       <c r="C191" t="n">
         <v>206.8385664547524</v>
@@ -5395,7 +5387,7 @@
         <v>203.2126188059985</v>
       </c>
       <c r="E191" t="n">
-        <v>204.9606628417969</v>
+        <v>204.6310298517525</v>
       </c>
       <c r="F191" t="n">
         <v>112001800</v>
@@ -5412,7 +5404,7 @@
         <v>46188</v>
       </c>
       <c r="B192" t="n">
-        <v>208.6864864049894</v>
+        <v>212.2125396728516</v>
       </c>
       <c r="C192" t="n">
         <v>212.4722588232193</v>
@@ -5421,7 +5413,7 @@
         <v>208.1071328472061</v>
       </c>
       <c r="E192" t="n">
-        <v>212.2125396728516</v>
+        <v>208.6864864049894</v>
       </c>
       <c r="F192" t="n">
         <v>149936700</v>
@@ -5438,7 +5430,7 @@
         <v>46189</v>
       </c>
       <c r="B193" t="n">
-        <v>210.9439520928381</v>
+        <v>207.1781768798828</v>
       </c>
       <c r="C193" t="n">
         <v>211.2536184019877</v>
@@ -5447,7 +5439,7 @@
         <v>207.0583006421773</v>
       </c>
       <c r="E193" t="n">
-        <v>207.1781768798828</v>
+        <v>210.9439520928381</v>
       </c>
       <c r="F193" t="n">
         <v>125694100</v>
@@ -5464,7 +5456,7 @@
         <v>46190</v>
       </c>
       <c r="B194" t="n">
-        <v>208.2969174543329</v>
+        <v>204.4212493896484</v>
       </c>
       <c r="C194" t="n">
         <v>208.9761653200819</v>
@@ -5473,7 +5465,7 @@
         <v>202.8530121596522</v>
       </c>
       <c r="E194" t="n">
-        <v>204.4212493896484</v>
+        <v>208.2969174543329</v>
       </c>
       <c r="F194" t="n">
         <v>128363500</v>
@@ -5490,7 +5482,7 @@
         <v>46191</v>
       </c>
       <c r="B195" t="n">
-        <v>207.0982684229139</v>
+        <v>210.4545135498047</v>
       </c>
       <c r="C195" t="n">
         <v>211.1537281092123</v>
@@ -5499,7 +5491,7 @@
         <v>206.2691942875683</v>
       </c>
       <c r="E195" t="n">
-        <v>210.4545135498047</v>
+        <v>207.0982684229139</v>
       </c>
       <c r="F195" t="n">
         <v>241272000</v>
@@ -5516,7 +5508,7 @@
         <v>46195</v>
       </c>
       <c r="B196" t="n">
-        <v>211.2036686200953</v>
+        <v>208.4167785644531</v>
       </c>
       <c r="C196" t="n">
         <v>213.7508214450341</v>
@@ -5525,7 +5517,7 @@
         <v>207.4878253737282</v>
       </c>
       <c r="E196" t="n">
-        <v>208.4167785644531</v>
+        <v>211.2036686200953</v>
       </c>
       <c r="F196" t="n">
         <v>122041400</v>
@@ -5542,7 +5534,7 @@
         <v>46196</v>
       </c>
       <c r="B197" t="n">
-        <v>201.9440304014853</v>
+        <v>199.81640625</v>
       </c>
       <c r="C197" t="n">
         <v>203.5422481594977</v>
@@ -5551,7 +5543,7 @@
         <v>199.77645766483</v>
       </c>
       <c r="E197" t="n">
-        <v>199.81640625</v>
+        <v>201.9440304014853</v>
       </c>
       <c r="F197" t="n">
         <v>153496200</v>
@@ -5568,7 +5560,7 @@
         <v>46197</v>
       </c>
       <c r="B198" t="n">
-        <v>199.8963159019567</v>
+        <v>198.7775726318359</v>
       </c>
       <c r="C198" t="n">
         <v>201.4445864758279</v>
@@ -5577,7 +5569,7 @@
         <v>196.360279356477</v>
       </c>
       <c r="E198" t="n">
-        <v>198.7775726318359</v>
+        <v>199.8963159019567</v>
       </c>
       <c r="F198" t="n">
         <v>151810700</v>
@@ -5594,7 +5586,7 @@
         <v>46198</v>
       </c>
       <c r="B199" t="n">
-        <v>199.8563704571445</v>
+        <v>195.5212249755859</v>
       </c>
       <c r="C199" t="n">
         <v>200.5755669254449</v>
@@ -5603,7 +5595,7 @@
         <v>191.9152592982058</v>
       </c>
       <c r="E199" t="n">
-        <v>195.5212249755859</v>
+        <v>199.8563704571445</v>
       </c>
       <c r="F199" t="n">
         <v>149550000</v>
@@ -5620,7 +5612,7 @@
         <v>46199</v>
       </c>
       <c r="B200" t="n">
-        <v>192.9041409641119</v>
+        <v>192.3148040771484</v>
       </c>
       <c r="C200" t="n">
         <v>195.331432829306</v>
@@ -5629,7 +5621,7 @@
         <v>191.0062707295152</v>
       </c>
       <c r="E200" t="n">
-        <v>192.3148040771484</v>
+        <v>192.9041409641119</v>
       </c>
       <c r="F200" t="n">
         <v>179304100</v>
@@ -5646,7 +5638,7 @@
         <v>46202</v>
       </c>
       <c r="B201" t="n">
-        <v>193.6333319429392</v>
+        <v>194.7520751953125</v>
       </c>
       <c r="C201" t="n">
         <v>195.9607141929515</v>
@@ -5655,7 +5647,7 @@
         <v>189.5878557469149</v>
       </c>
       <c r="E201" t="n">
-        <v>194.7520751953125</v>
+        <v>193.6333319429392</v>
       </c>
       <c r="F201" t="n">
         <v>148835700</v>
@@ -5672,7 +5664,7 @@
         <v>46203</v>
       </c>
       <c r="B202" t="n">
-        <v>197.0195429632178</v>
+        <v>199.8663482666016</v>
       </c>
       <c r="C202" t="n">
         <v>200.4057532237791</v>
@@ -5681,7 +5673,7 @@
         <v>194.8919188665145</v>
       </c>
       <c r="E202" t="n">
-        <v>199.8663482666016</v>
+        <v>197.0195429632178</v>
       </c>
       <c r="F202" t="n">
         <v>166476700</v>
@@ -5698,7 +5690,7 @@
         <v>46204</v>
       </c>
       <c r="B203" t="n">
-        <v>195.9806989625188</v>
+        <v>197.3591613769531</v>
       </c>
       <c r="C203" t="n">
         <v>199.626628404907</v>
@@ -5707,7 +5699,7 @@
         <v>193.2337727110923</v>
       </c>
       <c r="E203" t="n">
-        <v>197.3591613769531</v>
+        <v>195.9806989625188</v>
       </c>
       <c r="F203" t="n">
         <v>146147600</v>
@@ -5724,7 +5716,7 @@
         <v>46205</v>
       </c>
       <c r="B204" t="n">
-        <v>196.9196593659626</v>
+        <v>194.6122436523438</v>
       </c>
       <c r="C204" t="n">
         <v>199.8363939026278</v>
@@ -5733,7 +5725,7 @@
         <v>192.1350197738411</v>
       </c>
       <c r="E204" t="n">
-        <v>194.6122436523438</v>
+        <v>196.9196593659626</v>
       </c>
       <c r="F204" t="n">
         <v>142068700</v>
@@ -5750,7 +5742,7 @@
         <v>46209</v>
       </c>
       <c r="B205" t="n">
-        <v>194.202694284663</v>
+        <v>195.3314361572266</v>
       </c>
       <c r="C205" t="n">
         <v>197.3292007505161</v>
@@ -5759,7 +5751,7 @@
         <v>193.7731822131383</v>
       </c>
       <c r="E205" t="n">
-        <v>195.3314361572266</v>
+        <v>194.202694284663</v>
       </c>
       <c r="F205" t="n">
         <v>108999000</v>
@@ -5776,7 +5768,7 @@
         <v>46210</v>
       </c>
       <c r="B206" t="n">
-        <v>192.1549837798622</v>
+        <v>196.7098846435547</v>
       </c>
       <c r="C206" t="n">
         <v>198.1882414262674</v>
@@ -5785,7 +5777,7 @@
         <v>190.9263628146717</v>
       </c>
       <c r="E206" t="n">
-        <v>196.7098846435547</v>
+        <v>192.1549837798622</v>
       </c>
       <c r="F206" t="n">
         <v>124154600</v>
@@ -5802,7 +5794,7 @@
         <v>46211</v>
       </c>
       <c r="B207" t="n">
-        <v>194.9618356993413</v>
+        <v>203.891845703125</v>
       </c>
       <c r="C207" t="n">
         <v>204.9306918075912</v>
@@ -5811,7 +5803,7 @@
         <v>194.841974703339</v>
       </c>
       <c r="E207" t="n">
-        <v>203.891845703125</v>
+        <v>194.9618356993413</v>
       </c>
       <c r="F207" t="n">
         <v>147419100</v>
@@ -5828,7 +5820,7 @@
         <v>46212</v>
       </c>
       <c r="B208" t="n">
-        <v>204.2314748595287</v>
+        <v>202.5533447265625</v>
       </c>
       <c r="C208" t="n">
         <v>204.3613191897594</v>
@@ -5837,7 +5829,7 @@
         <v>198.7376223952696</v>
       </c>
       <c r="E208" t="n">
-        <v>202.5533447265625</v>
+        <v>204.2314748595287</v>
       </c>
       <c r="F208" t="n">
         <v>132037400</v>
@@ -5854,7 +5846,7 @@
         <v>46213</v>
       </c>
       <c r="B209" t="n">
-        <v>201.7742207048944</v>
+        <v>210.7242126464844</v>
       </c>
       <c r="C209" t="n">
         <v>210.7641612313501</v>
@@ -5863,7 +5855,7 @@
         <v>201.6943082934289</v>
       </c>
       <c r="E209" t="n">
-        <v>210.7242126464844</v>
+        <v>201.7742207048944</v>
       </c>
       <c r="F209" t="n">
         <v>148421000</v>
@@ -5880,7 +5872,7 @@
         <v>46216</v>
       </c>
       <c r="B210" t="n">
-        <v>208.3069001369788</v>
+        <v>203.3025054931641</v>
       </c>
       <c r="C210" t="n">
         <v>210.3346451505122</v>
@@ -5889,7 +5881,7 @@
         <v>202.7730991138312</v>
       </c>
       <c r="E210" t="n">
-        <v>203.3025054931641</v>
+        <v>208.3069001369788</v>
       </c>
       <c r="F210" t="n">
         <v>121411000</v>
@@ -5906,7 +5898,7 @@
         <v>46217</v>
       </c>
       <c r="B211" t="n">
-        <v>207.9672957533915</v>
+        <v>211.5632781982422</v>
       </c>
       <c r="C211" t="n">
         <v>212.3124399374416</v>
@@ -5915,7 +5907,7 @@
         <v>203.5722196467825</v>
       </c>
       <c r="E211" t="n">
-        <v>211.5632781982422</v>
+        <v>207.9672957533915</v>
       </c>
       <c r="F211" t="n">
         <v>124379600</v>
@@ -5932,7 +5924,7 @@
         <v>46218</v>
       </c>
       <c r="B212" t="n">
-        <v>211.7230919717581</v>
+        <v>212.2624816894531</v>
       </c>
       <c r="C212" t="n">
         <v>213.5710150202495</v>
@@ -5941,7 +5933,7 @@
         <v>205.8096955397309</v>
       </c>
       <c r="E212" t="n">
-        <v>212.2624816894531</v>
+        <v>211.7230919717581</v>
       </c>
       <c r="F212" t="n">
         <v>124797200</v>
@@ -5958,7 +5950,7 @@
         <v>46219</v>
       </c>
       <c r="B213" t="n">
-        <v>209.9350906043833</v>
+        <v>207.1681823730469</v>
       </c>
       <c r="C213" t="n">
         <v>210.8440771529852</v>
@@ -5967,7 +5959,7 @@
         <v>205.6199270055466</v>
       </c>
       <c r="E213" t="n">
-        <v>207.1681823730469</v>
+        <v>209.9350906043833</v>
       </c>
       <c r="F213" t="n">
         <v>122986100</v>
@@ -5984,7 +5976,7 @@
         <v>46220</v>
       </c>
       <c r="B214" t="n">
-        <v>202.4135048295048</v>
+        <v>202.5833129882812</v>
       </c>
       <c r="C214" t="n">
         <v>206.4190172896336</v>
@@ -5993,7 +5985,7 @@
         <v>197.7487264058434</v>
       </c>
       <c r="E214" t="n">
-        <v>202.5833129882812</v>
+        <v>202.4135048295048</v>
       </c>
       <c r="F214" t="n">
         <v>144281900</v>
@@ -6010,7 +6002,7 @@
         <v>46223</v>
       </c>
       <c r="B215" t="n">
-        <v>205.639896943356</v>
+        <v>203.0527954101562</v>
       </c>
       <c r="C215" t="n">
         <v>207.5078172334397</v>
@@ -6019,7 +6011,7 @@
         <v>202.0539130969454</v>
       </c>
       <c r="E215" t="n">
-        <v>203.0527954101562</v>
+        <v>205.639896943356</v>
       </c>
       <c r="F215" t="n">
         <v>88701500</v>
@@ -6036,7 +6028,7 @@
         <v>46224</v>
       </c>
       <c r="B216" t="n">
-        <v>207.308024406286</v>
+        <v>207.0583038330078</v>
       </c>
       <c r="C216" t="n">
         <v>208.4167843613107</v>
@@ -6045,7 +6037,7 @@
         <v>203.7819711309363</v>
       </c>
       <c r="E216" t="n">
-        <v>207.0583038330078</v>
+        <v>207.308024406286</v>
       </c>
       <c r="F216" t="n">
         <v>108685600</v>
@@ -6062,7 +6054,7 @@
         <v>46225</v>
       </c>
       <c r="B217" t="n">
-        <v>205.579968274895</v>
+        <v>211.8229827880859</v>
       </c>
       <c r="C217" t="n">
         <v>214.1503804276117</v>
@@ -6071,7 +6063,7 @@
         <v>204.7209288682105</v>
       </c>
       <c r="E217" t="n">
-        <v>211.8229827880859</v>
+        <v>205.579968274895</v>
       </c>
       <c r="F217" t="n">
         <v>137645600</v>
@@ -6088,7 +6080,7 @@
         <v>46226</v>
       </c>
       <c r="B218" t="n">
-        <v>209.2258868865651</v>
+        <v>208.5266571044922</v>
       </c>
       <c r="C218" t="n">
         <v>210.6342993029147</v>
@@ -6097,7 +6089,7 @@
         <v>205.7297989431358</v>
       </c>
       <c r="E218" t="n">
-        <v>208.5266571044922</v>
+        <v>209.2258868865651</v>
       </c>
       <c r="F218" t="n">
         <v>110505300</v>
@@ -6114,7 +6106,7 @@
         <v>46227</v>
       </c>
       <c r="B219" t="n">
-        <v>207.2181292349697</v>
+        <v>206.6088104248047</v>
       </c>
       <c r="C219" t="n">
         <v>211.6731509810223</v>
@@ -6123,7 +6115,7 @@
         <v>204.5810805834776</v>
       </c>
       <c r="E219" t="n">
-        <v>206.6088104248047</v>
+        <v>207.2181292349697</v>
       </c>
       <c r="F219" t="n">
         <v>114836800</v>
@@ -6140,7 +6132,7 @@
         <v>46230</v>
       </c>
       <c r="B220" t="n">
-        <v>207.9672962732577</v>
+        <v>196.2903594970703</v>
       </c>
       <c r="C220" t="n">
         <v>208.5166845983908</v>
@@ -6149,7 +6141,7 @@
         <v>195.2215633388429</v>
       </c>
       <c r="E220" t="n">
-        <v>196.2903594970703</v>
+        <v>207.9672962732577</v>
       </c>
       <c r="F220" t="n">
         <v>154353700</v>
@@ -6166,7 +6158,7 @@
         <v>46231</v>
       </c>
       <c r="B221" t="n">
-        <v>194.782047001347</v>
+        <v>196.789794921875</v>
       </c>
       <c r="C221" t="n">
         <v>198.4779084345641</v>
@@ -6175,7 +6167,7 @@
         <v>192.5245785077403</v>
       </c>
       <c r="E221" t="n">
-        <v>196.789794921875</v>
+        <v>194.782047001347</v>
       </c>
       <c r="F221" t="n">
         <v>134111500</v>
@@ -6192,7 +6184,7 @@
         <v>46232</v>
       </c>
       <c r="B222" t="n">
-        <v>195.6311069684468</v>
+        <v>189.7976226806641</v>
       </c>
       <c r="C222" t="n">
         <v>196.8497446088402</v>
@@ -6201,7 +6193,7 @@
         <v>189.7976226806641</v>
       </c>
       <c r="E222" t="n">
-        <v>189.7976226806641</v>
+        <v>195.6311069684468</v>
       </c>
       <c r="F222" t="n">
         <v>147680800</v>
@@ -6218,7 +6210,7 @@
         <v>46233</v>
       </c>
       <c r="B223" t="n">
-        <v>193.2337718176948</v>
+        <v>194.8219909667969</v>
       </c>
       <c r="C223" t="n">
         <v>197.0295274868271</v>
@@ -6227,7 +6219,7 @@
         <v>191.3059363552755</v>
       </c>
       <c r="E223" t="n">
-        <v>194.8219909667969</v>
+        <v>193.2337718176948</v>
       </c>
       <c r="F223" t="n">
         <v>129010200</v>
@@ -6244,7 +6236,7 @@
         <v>46234</v>
       </c>
       <c r="B224" t="n">
-        <v>198.2182038580375</v>
+        <v>200.5256195068359</v>
       </c>
       <c r="C224" t="n">
         <v>201.7742223680242</v>
@@ -6253,7 +6245,7 @@
         <v>194.7320991825756</v>
       </c>
       <c r="E224" t="n">
-        <v>200.5256195068359</v>
+        <v>198.2182038580375</v>
       </c>
       <c r="F224" t="n">
         <v>139961200</v>
@@ -6270,7 +6262,7 @@
         <v>46237</v>
       </c>
       <c r="B225" t="n">
-        <v>197.4690486270115</v>
+        <v>206.4090423583984</v>
       </c>
       <c r="C225" t="n">
         <v>208.506701330784</v>
@@ -6279,7 +6271,7 @@
         <v>196.6299911347511</v>
       </c>
       <c r="E225" t="n">
-        <v>206.4090423583984</v>
+        <v>197.4690486270115</v>
       </c>
       <c r="F225" t="n">
         <v>128406900</v>
@@ -6296,7 +6288,7 @@
         <v>46238</v>
       </c>
       <c r="B226" t="n">
-        <v>211.0638257011038</v>
+        <v>211.7031097412109</v>
       </c>
       <c r="C226" t="n">
         <v>212.8218530009649</v>
@@ -6305,7 +6297,7 @@
         <v>208.8163406042335</v>
       </c>
       <c r="E226" t="n">
-        <v>211.7031097412109</v>
+        <v>211.0638257011038</v>
       </c>
       <c r="F226" t="n">
         <v>134922000</v>
@@ -6322,7 +6314,7 @@
         <v>46239</v>
       </c>
       <c r="B227" t="n">
-        <v>216.6176127852948</v>
+        <v>218.9749755859375</v>
       </c>
       <c r="C227" t="n">
         <v>221.9716224388697</v>
@@ -6331,7 +6323,7 @@
         <v>216.1581202281489</v>
       </c>
       <c r="E227" t="n">
-        <v>218.9749755859375</v>
+        <v>216.6176127852948</v>
       </c>
       <c r="F227" t="n">
         <v>158187400</v>
@@ -6348,7 +6340,7 @@
         <v>46240</v>
       </c>
       <c r="B228" t="n">
-        <v>221.2823935806188</v>
+        <v>218.7452392578125</v>
       </c>
       <c r="C228" t="n">
         <v>223.3800524967045</v>
@@ -6357,7 +6349,7 @@
         <v>216.7574580038405</v>
       </c>
       <c r="E228" t="n">
-        <v>218.7452392578125</v>
+        <v>221.2823935806188</v>
       </c>
       <c r="F228" t="n">
         <v>113940600</v>
@@ -6374,7 +6366,7 @@
         <v>46241</v>
       </c>
       <c r="B229" t="n">
-        <v>221.2923777041913</v>
+        <v>223.7096862792969</v>
       </c>
       <c r="C229" t="n">
         <v>224.5087799247126</v>
@@ -6383,7 +6375,7 @@
         <v>220.4133716458871</v>
       </c>
       <c r="E229" t="n">
-        <v>223.7096862792969</v>
+        <v>221.2923777041913</v>
       </c>
       <c r="F229" t="n">
         <v>105669400</v>
@@ -6400,7 +6392,7 @@
         <v>46244</v>
       </c>
       <c r="B230" t="n">
-        <v>223.1502910726907</v>
+        <v>217.3068389892578</v>
       </c>
       <c r="C230" t="n">
         <v>223.8894694330602</v>
@@ -6409,7 +6401,7 @@
         <v>216.5277120448001</v>
       </c>
       <c r="E230" t="n">
-        <v>217.3068389892578</v>
+        <v>223.1502910726907</v>
       </c>
       <c r="F230" t="n">
         <v>115846600</v>
@@ -6426,7 +6418,7 @@
         <v>46245</v>
       </c>
       <c r="B231" t="n">
-        <v>221.9216754142795</v>
+        <v>217.2568969726562</v>
       </c>
       <c r="C231" t="n">
         <v>221.9516406634887</v>
@@ -6435,7 +6427,7 @@
         <v>215.9583469538982</v>
       </c>
       <c r="E231" t="n">
-        <v>217.2568969726562</v>
+        <v>221.9216754142795</v>
       </c>
       <c r="F231" t="n">
         <v>101273100</v>
@@ -6452,7 +6444,7 @@
         <v>46246</v>
       </c>
       <c r="B232" t="n">
-        <v>220.7929293559802</v>
+        <v>223.8395233154297</v>
       </c>
       <c r="C232" t="n">
         <v>224.848404158734</v>
@@ -6461,7 +6453,7 @@
         <v>219.9538719106106</v>
       </c>
       <c r="E232" t="n">
-        <v>223.8395233154297</v>
+        <v>220.7929293559802</v>
       </c>
       <c r="F232" t="n">
         <v>108783600</v>
@@ -6478,7 +6470,7 @@
         <v>46247</v>
       </c>
       <c r="B233" t="n">
-        <v>224.8084500146858</v>
+        <v>225.0481872558594</v>
       </c>
       <c r="C233" t="n">
         <v>226.9760227961096</v>
@@ -6487,7 +6479,7 @@
         <v>223.4599680426375</v>
       </c>
       <c r="E233" t="n">
-        <v>225.0481872558594</v>
+        <v>224.8084500146858</v>
       </c>
       <c r="F233" t="n">
         <v>98867200</v>
@@ -6504,7 +6496,7 @@
         <v>46248</v>
       </c>
       <c r="B234" t="n">
-        <v>226.5165415533859</v>
+        <v>224.9083404541016</v>
       </c>
       <c r="C234" t="n">
         <v>227.2357380227387</v>
@@ -6513,7 +6505,7 @@
         <v>224.2490744835724</v>
       </c>
       <c r="E234" t="n">
-        <v>224.9083404541016</v>
+        <v>226.5165415533859</v>
       </c>
       <c r="F234" t="n">
         <v>75680900</v>
@@ -6530,7 +6522,7 @@
         <v>46251</v>
       </c>
       <c r="B235" t="n">
-        <v>225.7274161885591</v>
+        <v>224.7584991455078</v>
       </c>
       <c r="C235" t="n">
         <v>227.6652502746616</v>
@@ -6539,7 +6531,7 @@
         <v>224.6086728983284</v>
       </c>
       <c r="E235" t="n">
-        <v>224.7584991455078</v>
+        <v>225.7274161885591</v>
       </c>
       <c r="F235" t="n">
         <v>93678700</v>
@@ -6556,7 +6548,7 @@
         <v>46252</v>
       </c>
       <c r="B236" t="n">
-        <v>220.203597915372</v>
+        <v>219.4944000244141</v>
       </c>
       <c r="C236" t="n">
         <v>221.3922702798686</v>
@@ -6565,7 +6557,7 @@
         <v>218.4455705709327</v>
       </c>
       <c r="E236" t="n">
-        <v>219.4944000244141</v>
+        <v>220.203597915372</v>
       </c>
       <c r="F236" t="n">
         <v>103128200</v>
@@ -6582,7 +6574,7 @@
         <v>46253</v>
       </c>
       <c r="B237" t="n">
-        <v>221.4222404106533</v>
+        <v>217.3168334960938</v>
       </c>
       <c r="C237" t="n">
         <v>222.6208961374568</v>
@@ -6591,7 +6583,7 @@
         <v>216.5177245976465</v>
       </c>
       <c r="E237" t="n">
-        <v>217.3168334960938</v>
+        <v>221.4222404106533</v>
       </c>
       <c r="F237" t="n">
         <v>96797300</v>
@@ -6608,7 +6600,7 @@
         <v>46254</v>
       </c>
       <c r="B238" t="n">
-        <v>218.1159423024499</v>
+        <v>216.6076354980469</v>
       </c>
       <c r="C238" t="n">
         <v>219.6142657707553</v>
@@ -6617,7 +6609,7 @@
         <v>215.418963107847</v>
       </c>
       <c r="E238" t="n">
-        <v>216.6076354980469</v>
+        <v>218.1159423024499</v>
       </c>
       <c r="F238" t="n">
         <v>92457000</v>
@@ -6634,7 +6626,7 @@
         <v>46255</v>
       </c>
       <c r="B239" t="n">
-        <v>218.1758724878036</v>
+        <v>214.4800109863281</v>
       </c>
       <c r="C239" t="n">
         <v>218.4955221432803</v>
@@ -6643,7 +6635,7 @@
         <v>214.2602556586216</v>
       </c>
       <c r="E239" t="n">
-        <v>214.4800109863281</v>
+        <v>218.1758724878036</v>
       </c>
       <c r="F239" t="n">
         <v>98869300</v>
@@ -6660,7 +6652,7 @@
         <v>46258</v>
       </c>
       <c r="B240" t="n">
-        <v>215.2891020611033</v>
+        <v>208.2469787597656</v>
       </c>
       <c r="C240" t="n">
         <v>215.3490325607492</v>
@@ -6669,7 +6661,7 @@
         <v>207.0183577918231</v>
       </c>
       <c r="E240" t="n">
-        <v>208.2469787597656</v>
+        <v>215.2891020611033</v>
       </c>
       <c r="F240" t="n">
         <v>135187300</v>
@@ -6686,7 +6678,7 @@
         <v>46259</v>
       </c>
       <c r="B241" t="n">
-        <v>210.7941279013131</v>
+        <v>212.8118743896484</v>
       </c>
       <c r="C241" t="n">
         <v>214.4899893165327</v>
@@ -6695,7 +6687,7 @@
         <v>209.8751580258669</v>
       </c>
       <c r="E241" t="n">
-        <v>212.8118743896484</v>
+        <v>210.7941279013131</v>
       </c>
       <c r="F241" t="n">
         <v>122309000</v>
@@ -6712,7 +6704,7 @@
         <v>46260</v>
       </c>
       <c r="B242" t="n">
-        <v>212.4023240594531</v>
+        <v>209.4256591796875</v>
       </c>
       <c r="C242" t="n">
         <v>213.3612577394914</v>
@@ -6721,7 +6713,7 @@
         <v>208.9961318803605</v>
       </c>
       <c r="E242" t="n">
-        <v>209.4256591796875</v>
+        <v>212.4023240594531</v>
       </c>
       <c r="F242" t="n">
         <v>179900000</v>
@@ -6738,7 +6730,7 @@
         <v>46261</v>
       </c>
       <c r="B243" t="n">
-        <v>222.6109016432552</v>
+        <v>227.7251739501953</v>
       </c>
       <c r="C243" t="n">
         <v>230.2123962709879</v>
@@ -6747,7 +6739,7 @@
         <v>220.6530857022795</v>
       </c>
       <c r="E243" t="n">
-        <v>227.7251739501953</v>
+        <v>222.6109016432552</v>
       </c>
       <c r="F243" t="n">
         <v>298909800</v>
@@ -6764,7 +6756,7 @@
         <v>46262</v>
       </c>
       <c r="B244" t="n">
-        <v>227.1058715337123</v>
+        <v>217.3068389892578</v>
       </c>
       <c r="C244" t="n">
         <v>229.003741733446</v>
@@ -6773,7 +6765,7 @@
         <v>216.5676606288883</v>
       </c>
       <c r="E244" t="n">
-        <v>217.3068389892578</v>
+        <v>227.1058715337123</v>
       </c>
       <c r="F244" t="n">
         <v>195116400</v>
@@ -6790,7 +6782,7 @@
         <v>46265</v>
       </c>
       <c r="B245" t="n">
-        <v>218.6253647857836</v>
+        <v>220.5332336425781</v>
       </c>
       <c r="C245" t="n">
         <v>221.0526567078369</v>
@@ -6799,7 +6791,7 @@
         <v>215.9683494434545</v>
       </c>
       <c r="E245" t="n">
-        <v>220.5332336425781</v>
+        <v>218.6253647857836</v>
       </c>
       <c r="F245" t="n">
         <v>124702700</v>
@@ -6816,7 +6808,7 @@
         <v>46266</v>
       </c>
       <c r="B246" t="n">
-        <v>216.5077444634259</v>
+        <v>217.1969757080078</v>
       </c>
       <c r="C246" t="n">
         <v>220.1636574397174</v>
@@ -6825,7 +6817,7 @@
         <v>214.8595947199138</v>
       </c>
       <c r="E246" t="n">
-        <v>217.1969757080078</v>
+        <v>216.5077444634259</v>
       </c>
       <c r="F246" t="n">
         <v>109756200</v>
@@ -6842,7 +6834,7 @@
         <v>46267</v>
       </c>
       <c r="B247" t="n">
-        <v>218.5454508199983</v>
+        <v>224.1591796875</v>
       </c>
       <c r="C247" t="n">
         <v>227.6952163087265</v>
@@ -6851,7 +6843,7 @@
         <v>218.2357997469377</v>
       </c>
       <c r="E247" t="n">
-        <v>224.1591796875</v>
+        <v>218.5454508199983</v>
       </c>
       <c r="F247" t="n">
         <v>157104700</v>
@@ -6868,7 +6860,7 @@
         <v>46268</v>
       </c>
       <c r="B248" t="n">
-        <v>225.7673797205316</v>
+        <v>228.1946563720703</v>
       </c>
       <c r="C248" t="n">
         <v>230.1424737915274</v>
@@ -6877,7 +6869,7 @@
         <v>224.4987949430455</v>
       </c>
       <c r="E248" t="n">
-        <v>228.1946563720703</v>
+        <v>225.7673797205316</v>
       </c>
       <c r="F248" t="n">
         <v>134681600</v>
@@ -6894,7 +6886,7 @@
         <v>46269</v>
       </c>
       <c r="B249" t="n">
-        <v>230.8317036041433</v>
+        <v>230.1025238037109</v>
       </c>
       <c r="C249" t="n">
         <v>234.4975997614268</v>
@@ -6903,7 +6895,7 @@
         <v>229.3733440032785</v>
       </c>
       <c r="E249" t="n">
-        <v>230.1025238037109</v>
+        <v>230.8317036041433</v>
       </c>
       <c r="F249" t="n">
         <v>135352400</v>
@@ -6920,7 +6912,7 @@
         <v>46273</v>
       </c>
       <c r="B250" t="n">
-        <v>232.8494477166676</v>
+        <v>225.4776916503906</v>
       </c>
       <c r="C250" t="n">
         <v>233.4487831783142</v>
@@ -6929,7 +6921,7 @@
         <v>224.5986856128386</v>
       </c>
       <c r="E250" t="n">
-        <v>225.4776916503906</v>
+        <v>232.8494477166676</v>
       </c>
       <c r="F250" t="n">
         <v>122965600</v>
@@ -6946,7 +6938,7 @@
         <v>46274</v>
       </c>
       <c r="B251" t="n">
-        <v>225.0281992525124</v>
+        <v>223.4199981689453</v>
       </c>
       <c r="C251" t="n">
         <v>225.9271872095504</v>
@@ -6955,7 +6947,7 @@
         <v>223.2102414251123</v>
       </c>
       <c r="E251" t="n">
-        <v>223.4199981689453</v>
+        <v>225.0281992525124</v>
       </c>
       <c r="F251" t="n">
         <v>82955500</v>
@@ -6972,7 +6964,7 @@
         <v>46275</v>
       </c>
       <c r="B252" t="n">
-        <v>220.5299987792969</v>
+        <v>218.3600006103516</v>
       </c>
       <c r="C252" t="n">
         <v>220.9900054931641</v>
@@ -6981,15 +6973,41 @@
         <v>217.1999969482422</v>
       </c>
       <c r="E252" t="n">
-        <v>218.3600006103516</v>
+        <v>220.5299987792969</v>
       </c>
       <c r="F252" t="n">
-        <v>105482000</v>
+        <v>105768000</v>
       </c>
       <c r="G252" t="n">
         <v>0.25</v>
       </c>
       <c r="H252" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="1" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B253" t="n">
+        <v>218.2899932861328</v>
+      </c>
+      <c r="C253" t="n">
+        <v>222</v>
+      </c>
+      <c r="D253" t="n">
+        <v>218.1499938964844</v>
+      </c>
+      <c r="E253" t="n">
+        <v>221.2400054931641</v>
+      </c>
+      <c r="F253" t="n">
+        <v>88804100</v>
+      </c>
+      <c r="G253" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10884,37 +10902,37 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>218.29</v>
+      </c>
+      <c r="D2" t="n">
         <v>218.36</v>
       </c>
-      <c r="D2" t="n">
-        <v>223.67</v>
-      </c>
       <c r="E2" t="n">
-        <v>220.485</v>
+        <v>221.25</v>
       </c>
       <c r="F2" t="n">
-        <v>220.99</v>
+        <v>222</v>
       </c>
       <c r="G2" t="n">
-        <v>217.2</v>
+        <v>218.15</v>
       </c>
       <c r="H2" t="n">
-        <v>100845811</v>
+        <v>86818741</v>
       </c>
       <c r="I2" t="n">
-        <v>132898814</v>
+        <v>132087064</v>
       </c>
       <c r="J2" t="n">
-        <v>5272738725888</v>
+        <v>5271048421376</v>
       </c>
       <c r="K2" t="n">
-        <v>27.640507</v>
+        <v>27.631645</v>
       </c>
       <c r="L2" t="n">
-        <v>14.026631</v>
+        <v>14.022135</v>
       </c>
       <c r="M2" t="n">
-        <v>7.73</v>
+        <v>7.9</v>
       </c>
       <c r="N2" t="n">
         <v>236.54</v>
@@ -10950,7 +10968,7 @@
         <v>9.483000000000001</v>
       </c>
       <c r="Y2" t="n">
-        <v>23.026468</v>
+        <v>23.019087</v>
       </c>
       <c r="Z2" t="n">
         <v>1.278</v>
@@ -10962,7 +10980,7 @@
         <v>302970011648</v>
       </c>
       <c r="AC2" t="n">
-        <v>5238867099648</v>
+        <v>5237179940864</v>
       </c>
       <c r="AD2" t="n">
         <v>201266003968</v>
@@ -10989,7 +11007,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-11 19:02:59</t>
+          <t>2026-09-12 21:47:03</t>
         </is>
       </c>
     </row>

</xml_diff>